<commit_message>
feat: populate purchase orders table with live commercial orders and payments due (.815M) and add process payment workflow
</commit_message>
<xml_diff>
--- a/KSBC_Banking_ERP_Master_Data.xlsx
+++ b/KSBC_Banking_ERP_Master_Data.xlsx
@@ -448,7 +448,7 @@
         <v>Active</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-07-29T15:27:01.498Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="3">
@@ -471,7 +471,7 @@
         <v>Active</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-07-29T15:27:01.498Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="4">
@@ -494,7 +494,7 @@
         <v>Active</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-07-29T15:27:01.498Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="5">
@@ -517,7 +517,7 @@
         <v>Active</v>
       </c>
       <c r="G5" t="str">
-        <v>2026-07-29T15:27:01.498Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="6">
@@ -540,7 +540,7 @@
         <v>Active</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-07-29T15:27:01.498Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="7">
@@ -563,7 +563,7 @@
         <v>Active</v>
       </c>
       <c r="G7" t="str">
-        <v>2026-07-29T15:27:01.498Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="8">
@@ -586,7 +586,7 @@
         <v>Active</v>
       </c>
       <c r="G8" t="str">
-        <v>2026-07-29T15:27:01.498Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
   </sheetData>
@@ -679,7 +679,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M2" t="str">
-        <v>2025-12-22T15:27:01.498Z</v>
+        <v>2025-12-23T15:50:37.934Z</v>
       </c>
     </row>
     <row r="3">
@@ -720,7 +720,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M3" t="str">
-        <v>2025-12-23T15:27:01.498Z</v>
+        <v>2025-12-24T15:50:37.934Z</v>
       </c>
     </row>
     <row r="4">
@@ -761,7 +761,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M4" t="str">
-        <v>2025-12-24T15:27:01.498Z</v>
+        <v>2025-12-25T15:50:37.934Z</v>
       </c>
     </row>
     <row r="5">
@@ -802,7 +802,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M5" t="str">
-        <v>2025-12-25T15:27:01.498Z</v>
+        <v>2025-12-26T15:50:37.934Z</v>
       </c>
     </row>
     <row r="6">
@@ -843,7 +843,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M6" t="str">
-        <v>2025-12-26T15:27:01.498Z</v>
+        <v>2025-12-27T15:50:37.934Z</v>
       </c>
     </row>
     <row r="7">
@@ -884,7 +884,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M7" t="str">
-        <v>2025-12-27T15:27:01.498Z</v>
+        <v>2025-12-28T15:50:37.934Z</v>
       </c>
     </row>
     <row r="8">
@@ -925,7 +925,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M8" t="str">
-        <v>2025-12-28T15:27:01.498Z</v>
+        <v>2025-12-29T15:50:37.934Z</v>
       </c>
     </row>
     <row r="9">
@@ -966,7 +966,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M9" t="str">
-        <v>2025-12-29T15:27:01.498Z</v>
+        <v>2025-12-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="10">
@@ -1007,7 +1007,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M10" t="str">
-        <v>2025-12-30T15:27:01.498Z</v>
+        <v>2025-12-31T15:50:37.934Z</v>
       </c>
     </row>
     <row r="11">
@@ -1048,7 +1048,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M11" t="str">
-        <v>2025-12-31T15:27:01.498Z</v>
+        <v>2026-01-01T15:50:37.934Z</v>
       </c>
     </row>
     <row r="12">
@@ -1089,7 +1089,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M12" t="str">
-        <v>2026-01-01T15:27:01.498Z</v>
+        <v>2026-01-02T15:50:37.934Z</v>
       </c>
     </row>
     <row r="13">
@@ -1130,7 +1130,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M13" t="str">
-        <v>2026-01-02T15:27:01.498Z</v>
+        <v>2026-01-03T15:50:37.934Z</v>
       </c>
     </row>
     <row r="14">
@@ -1171,7 +1171,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M14" t="str">
-        <v>2026-01-03T15:27:01.498Z</v>
+        <v>2026-01-04T15:50:37.934Z</v>
       </c>
     </row>
     <row r="15">
@@ -1212,7 +1212,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M15" t="str">
-        <v>2026-01-04T15:27:01.498Z</v>
+        <v>2026-01-05T15:50:37.934Z</v>
       </c>
     </row>
     <row r="16">
@@ -1253,7 +1253,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M16" t="str">
-        <v>2026-01-05T15:27:01.498Z</v>
+        <v>2026-01-06T15:50:37.934Z</v>
       </c>
     </row>
     <row r="17">
@@ -1294,7 +1294,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M17" t="str">
-        <v>2026-01-06T15:27:01.498Z</v>
+        <v>2026-01-07T15:50:37.934Z</v>
       </c>
     </row>
     <row r="18">
@@ -1335,7 +1335,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M18" t="str">
-        <v>2026-01-07T15:27:01.498Z</v>
+        <v>2026-01-08T15:50:37.934Z</v>
       </c>
     </row>
     <row r="19">
@@ -1376,7 +1376,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M19" t="str">
-        <v>2026-01-08T15:27:01.498Z</v>
+        <v>2026-01-09T15:50:37.934Z</v>
       </c>
     </row>
     <row r="20">
@@ -1417,7 +1417,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M20" t="str">
-        <v>2026-01-09T15:27:01.498Z</v>
+        <v>2026-01-10T15:50:37.934Z</v>
       </c>
     </row>
     <row r="21">
@@ -1458,7 +1458,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M21" t="str">
-        <v>2026-01-10T15:27:01.498Z</v>
+        <v>2026-01-11T15:50:37.934Z</v>
       </c>
     </row>
     <row r="22">
@@ -1499,7 +1499,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M22" t="str">
-        <v>2026-01-11T15:27:01.498Z</v>
+        <v>2026-01-12T15:50:37.934Z</v>
       </c>
     </row>
     <row r="23">
@@ -1540,7 +1540,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M23" t="str">
-        <v>2026-01-12T15:27:01.498Z</v>
+        <v>2026-01-13T15:50:37.934Z</v>
       </c>
     </row>
     <row r="24">
@@ -1581,7 +1581,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M24" t="str">
-        <v>2026-01-13T15:27:01.498Z</v>
+        <v>2026-01-14T15:50:37.934Z</v>
       </c>
     </row>
     <row r="25">
@@ -1622,7 +1622,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M25" t="str">
-        <v>2026-01-14T15:27:01.498Z</v>
+        <v>2026-01-15T15:50:37.934Z</v>
       </c>
     </row>
     <row r="26">
@@ -1663,7 +1663,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M26" t="str">
-        <v>2026-01-15T15:27:01.498Z</v>
+        <v>2026-01-16T15:50:37.934Z</v>
       </c>
     </row>
     <row r="27">
@@ -1704,7 +1704,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M27" t="str">
-        <v>2026-01-16T15:27:01.498Z</v>
+        <v>2026-01-17T15:50:37.934Z</v>
       </c>
     </row>
     <row r="28">
@@ -1745,7 +1745,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M28" t="str">
-        <v>2026-01-17T15:27:01.498Z</v>
+        <v>2026-01-18T15:50:37.934Z</v>
       </c>
     </row>
     <row r="29">
@@ -1786,7 +1786,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M29" t="str">
-        <v>2026-01-18T15:27:01.498Z</v>
+        <v>2026-01-19T15:50:37.934Z</v>
       </c>
     </row>
     <row r="30">
@@ -1827,7 +1827,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M30" t="str">
-        <v>2026-01-19T15:27:01.498Z</v>
+        <v>2026-01-20T15:50:37.934Z</v>
       </c>
     </row>
     <row r="31">
@@ -1868,7 +1868,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M31" t="str">
-        <v>2026-01-20T15:27:01.498Z</v>
+        <v>2026-01-21T15:50:37.934Z</v>
       </c>
     </row>
     <row r="32">
@@ -1909,7 +1909,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M32" t="str">
-        <v>2026-01-21T15:27:01.498Z</v>
+        <v>2026-01-22T15:50:37.935Z</v>
       </c>
     </row>
     <row r="33">
@@ -1950,7 +1950,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M33" t="str">
-        <v>2026-01-22T15:27:01.498Z</v>
+        <v>2026-01-23T15:50:37.935Z</v>
       </c>
     </row>
     <row r="34">
@@ -1991,7 +1991,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M34" t="str">
-        <v>2026-01-23T15:27:01.498Z</v>
+        <v>2026-01-24T15:50:37.935Z</v>
       </c>
     </row>
     <row r="35">
@@ -2032,7 +2032,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M35" t="str">
-        <v>2026-01-24T15:27:01.498Z</v>
+        <v>2026-01-25T15:50:37.935Z</v>
       </c>
     </row>
     <row r="36">
@@ -2073,7 +2073,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M36" t="str">
-        <v>2026-01-25T15:27:01.498Z</v>
+        <v>2026-01-26T15:50:37.935Z</v>
       </c>
     </row>
     <row r="37">
@@ -2114,7 +2114,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M37" t="str">
-        <v>2026-01-26T15:27:01.498Z</v>
+        <v>2026-01-27T15:50:37.935Z</v>
       </c>
     </row>
     <row r="38">
@@ -2155,7 +2155,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M38" t="str">
-        <v>2026-01-27T15:27:01.498Z</v>
+        <v>2026-01-28T15:50:37.935Z</v>
       </c>
     </row>
     <row r="39">
@@ -2196,7 +2196,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M39" t="str">
-        <v>2026-01-28T15:27:01.498Z</v>
+        <v>2026-01-29T15:50:37.935Z</v>
       </c>
     </row>
     <row r="40">
@@ -2237,7 +2237,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M40" t="str">
-        <v>2026-01-29T15:27:01.498Z</v>
+        <v>2026-01-30T15:50:37.935Z</v>
       </c>
     </row>
     <row r="41">
@@ -2278,7 +2278,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M41" t="str">
-        <v>2026-01-30T15:27:01.498Z</v>
+        <v>2026-01-31T15:50:37.935Z</v>
       </c>
     </row>
     <row r="42">
@@ -2319,7 +2319,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M42" t="str">
-        <v>2026-01-31T15:27:01.498Z</v>
+        <v>2026-02-01T15:50:37.935Z</v>
       </c>
     </row>
     <row r="43">
@@ -2360,7 +2360,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M43" t="str">
-        <v>2026-02-01T15:27:01.498Z</v>
+        <v>2026-02-02T15:50:37.935Z</v>
       </c>
     </row>
     <row r="44">
@@ -2401,7 +2401,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M44" t="str">
-        <v>2026-02-02T15:27:01.498Z</v>
+        <v>2026-02-03T15:50:37.935Z</v>
       </c>
     </row>
     <row r="45">
@@ -2442,7 +2442,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M45" t="str">
-        <v>2026-02-03T15:27:01.498Z</v>
+        <v>2026-02-04T15:50:37.935Z</v>
       </c>
     </row>
     <row r="46">
@@ -2483,7 +2483,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M46" t="str">
-        <v>2026-02-04T15:27:01.498Z</v>
+        <v>2026-02-05T15:50:37.935Z</v>
       </c>
     </row>
     <row r="47">
@@ -2524,7 +2524,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M47" t="str">
-        <v>2026-02-05T15:27:01.498Z</v>
+        <v>2026-02-06T15:50:37.935Z</v>
       </c>
     </row>
     <row r="48">
@@ -2565,7 +2565,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M48" t="str">
-        <v>2026-02-06T15:27:01.498Z</v>
+        <v>2026-02-07T15:50:37.935Z</v>
       </c>
     </row>
     <row r="49">
@@ -2606,7 +2606,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M49" t="str">
-        <v>2026-02-07T15:27:01.498Z</v>
+        <v>2026-02-08T15:50:37.935Z</v>
       </c>
     </row>
     <row r="50">
@@ -2647,7 +2647,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M50" t="str">
-        <v>2026-02-08T15:27:01.498Z</v>
+        <v>2026-02-09T15:50:37.935Z</v>
       </c>
     </row>
     <row r="51">
@@ -2688,7 +2688,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M51" t="str">
-        <v>2026-02-09T15:27:01.498Z</v>
+        <v>2026-02-10T15:50:37.935Z</v>
       </c>
     </row>
     <row r="52">
@@ -2729,7 +2729,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M52" t="str">
-        <v>2026-02-10T15:27:01.498Z</v>
+        <v>2026-02-11T15:50:37.935Z</v>
       </c>
     </row>
     <row r="53">
@@ -2770,7 +2770,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M53" t="str">
-        <v>2026-02-11T15:27:01.498Z</v>
+        <v>2026-02-12T15:50:37.935Z</v>
       </c>
     </row>
     <row r="54">
@@ -2811,7 +2811,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M54" t="str">
-        <v>2026-02-12T15:27:01.498Z</v>
+        <v>2026-02-13T15:50:37.935Z</v>
       </c>
     </row>
     <row r="55">
@@ -2852,7 +2852,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M55" t="str">
-        <v>2026-02-13T15:27:01.499Z</v>
+        <v>2026-02-14T15:50:37.935Z</v>
       </c>
     </row>
     <row r="56">
@@ -2893,7 +2893,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M56" t="str">
-        <v>2026-02-14T15:27:01.499Z</v>
+        <v>2026-02-15T15:50:37.935Z</v>
       </c>
     </row>
     <row r="57">
@@ -2934,7 +2934,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M57" t="str">
-        <v>2026-02-15T15:27:01.499Z</v>
+        <v>2026-02-16T15:50:37.935Z</v>
       </c>
     </row>
     <row r="58">
@@ -2975,7 +2975,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M58" t="str">
-        <v>2026-02-16T15:27:01.499Z</v>
+        <v>2026-02-17T15:50:37.935Z</v>
       </c>
     </row>
     <row r="59">
@@ -3016,7 +3016,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M59" t="str">
-        <v>2026-02-17T15:27:01.499Z</v>
+        <v>2026-02-18T15:50:37.935Z</v>
       </c>
     </row>
     <row r="60">
@@ -3057,7 +3057,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M60" t="str">
-        <v>2026-02-18T15:27:01.499Z</v>
+        <v>2026-02-19T15:50:37.935Z</v>
       </c>
     </row>
     <row r="61">
@@ -3098,7 +3098,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M61" t="str">
-        <v>2026-02-19T15:27:01.499Z</v>
+        <v>2026-02-20T15:50:37.935Z</v>
       </c>
     </row>
     <row r="62">
@@ -3139,7 +3139,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M62" t="str">
-        <v>2026-02-20T15:27:01.499Z</v>
+        <v>2026-02-21T15:50:37.935Z</v>
       </c>
     </row>
     <row r="63">
@@ -3180,7 +3180,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M63" t="str">
-        <v>2026-02-21T15:27:01.499Z</v>
+        <v>2026-02-22T15:50:37.935Z</v>
       </c>
     </row>
     <row r="64">
@@ -3221,7 +3221,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M64" t="str">
-        <v>2026-02-22T15:27:01.499Z</v>
+        <v>2026-02-23T15:50:37.935Z</v>
       </c>
     </row>
     <row r="65">
@@ -3262,7 +3262,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M65" t="str">
-        <v>2026-02-23T15:27:01.499Z</v>
+        <v>2026-02-24T15:50:37.935Z</v>
       </c>
     </row>
     <row r="66">
@@ -3303,7 +3303,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M66" t="str">
-        <v>2026-02-24T15:27:01.499Z</v>
+        <v>2026-02-25T15:50:37.935Z</v>
       </c>
     </row>
     <row r="67">
@@ -3344,7 +3344,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M67" t="str">
-        <v>2026-02-25T15:27:01.499Z</v>
+        <v>2026-02-26T15:50:37.935Z</v>
       </c>
     </row>
     <row r="68">
@@ -3385,7 +3385,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M68" t="str">
-        <v>2026-02-26T15:27:01.499Z</v>
+        <v>2026-02-27T15:50:37.935Z</v>
       </c>
     </row>
     <row r="69">
@@ -3426,7 +3426,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M69" t="str">
-        <v>2026-02-27T15:27:01.499Z</v>
+        <v>2026-02-28T15:50:37.935Z</v>
       </c>
     </row>
     <row r="70">
@@ -3467,7 +3467,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M70" t="str">
-        <v>2026-02-28T15:27:01.499Z</v>
+        <v>2026-03-01T15:50:37.935Z</v>
       </c>
     </row>
     <row r="71">
@@ -3508,7 +3508,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M71" t="str">
-        <v>2026-03-01T15:27:01.499Z</v>
+        <v>2026-03-02T15:50:37.935Z</v>
       </c>
     </row>
     <row r="72">
@@ -3549,7 +3549,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M72" t="str">
-        <v>2026-03-02T15:27:01.499Z</v>
+        <v>2026-03-03T15:50:37.935Z</v>
       </c>
     </row>
     <row r="73">
@@ -3590,7 +3590,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M73" t="str">
-        <v>2026-03-03T15:27:01.499Z</v>
+        <v>2026-03-04T15:50:37.935Z</v>
       </c>
     </row>
     <row r="74">
@@ -3631,7 +3631,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M74" t="str">
-        <v>2026-03-04T15:27:01.499Z</v>
+        <v>2026-03-05T15:50:37.935Z</v>
       </c>
     </row>
     <row r="75">
@@ -3672,7 +3672,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M75" t="str">
-        <v>2026-03-05T15:27:01.499Z</v>
+        <v>2026-03-06T15:50:37.935Z</v>
       </c>
     </row>
     <row r="76">
@@ -3713,7 +3713,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M76" t="str">
-        <v>2026-03-06T15:27:01.499Z</v>
+        <v>2026-03-07T15:50:37.935Z</v>
       </c>
     </row>
     <row r="77">
@@ -3754,7 +3754,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M77" t="str">
-        <v>2026-03-07T15:27:01.499Z</v>
+        <v>2026-03-08T15:50:37.935Z</v>
       </c>
     </row>
     <row r="78">
@@ -3795,7 +3795,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M78" t="str">
-        <v>2026-03-08T15:27:01.499Z</v>
+        <v>2026-03-09T15:50:37.935Z</v>
       </c>
     </row>
     <row r="79">
@@ -3836,7 +3836,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M79" t="str">
-        <v>2026-03-09T15:27:01.499Z</v>
+        <v>2026-03-10T15:50:37.935Z</v>
       </c>
     </row>
     <row r="80">
@@ -3877,7 +3877,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M80" t="str">
-        <v>2026-03-10T15:27:01.499Z</v>
+        <v>2026-03-11T15:50:37.935Z</v>
       </c>
     </row>
     <row r="81">
@@ -3918,7 +3918,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M81" t="str">
-        <v>2026-03-11T15:27:01.499Z</v>
+        <v>2026-03-12T15:50:37.935Z</v>
       </c>
     </row>
     <row r="82">
@@ -3959,7 +3959,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M82" t="str">
-        <v>2026-03-12T15:27:01.499Z</v>
+        <v>2026-03-13T15:50:37.935Z</v>
       </c>
     </row>
     <row r="83">
@@ -4000,7 +4000,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M83" t="str">
-        <v>2026-03-13T15:27:01.499Z</v>
+        <v>2026-03-14T15:50:37.935Z</v>
       </c>
     </row>
     <row r="84">
@@ -4041,7 +4041,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M84" t="str">
-        <v>2026-03-14T15:27:01.499Z</v>
+        <v>2026-03-15T15:50:37.935Z</v>
       </c>
     </row>
     <row r="85">
@@ -4082,7 +4082,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M85" t="str">
-        <v>2026-03-15T15:27:01.499Z</v>
+        <v>2026-03-16T15:50:37.935Z</v>
       </c>
     </row>
     <row r="86">
@@ -4123,7 +4123,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M86" t="str">
-        <v>2026-03-16T15:27:01.499Z</v>
+        <v>2026-03-17T15:50:37.935Z</v>
       </c>
     </row>
     <row r="87">
@@ -4164,7 +4164,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M87" t="str">
-        <v>2026-03-17T15:27:01.499Z</v>
+        <v>2026-03-18T15:50:37.935Z</v>
       </c>
     </row>
     <row r="88">
@@ -4205,7 +4205,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M88" t="str">
-        <v>2026-03-18T15:27:01.499Z</v>
+        <v>2026-03-19T15:50:37.935Z</v>
       </c>
     </row>
     <row r="89">
@@ -4246,7 +4246,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M89" t="str">
-        <v>2026-03-19T15:27:01.499Z</v>
+        <v>2026-03-20T15:50:37.935Z</v>
       </c>
     </row>
     <row r="90">
@@ -4287,7 +4287,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M90" t="str">
-        <v>2026-03-20T15:27:01.499Z</v>
+        <v>2026-03-21T15:50:37.935Z</v>
       </c>
     </row>
     <row r="91">
@@ -4328,7 +4328,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M91" t="str">
-        <v>2026-03-21T15:27:01.499Z</v>
+        <v>2026-03-22T15:50:37.935Z</v>
       </c>
     </row>
     <row r="92">
@@ -4369,7 +4369,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M92" t="str">
-        <v>2026-03-22T15:27:01.499Z</v>
+        <v>2026-03-23T15:50:37.935Z</v>
       </c>
     </row>
     <row r="93">
@@ -4410,7 +4410,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M93" t="str">
-        <v>2026-03-23T15:27:01.499Z</v>
+        <v>2026-03-24T15:50:37.935Z</v>
       </c>
     </row>
     <row r="94">
@@ -4451,7 +4451,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M94" t="str">
-        <v>2026-03-24T15:27:01.499Z</v>
+        <v>2026-03-25T15:50:37.935Z</v>
       </c>
     </row>
     <row r="95">
@@ -4492,7 +4492,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M95" t="str">
-        <v>2026-03-25T15:27:01.499Z</v>
+        <v>2026-03-26T15:50:37.935Z</v>
       </c>
     </row>
     <row r="96">
@@ -4533,7 +4533,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M96" t="str">
-        <v>2026-03-26T15:27:01.499Z</v>
+        <v>2026-03-27T15:50:37.935Z</v>
       </c>
     </row>
     <row r="97">
@@ -4574,7 +4574,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M97" t="str">
-        <v>2026-03-27T15:27:01.499Z</v>
+        <v>2026-03-28T15:50:37.935Z</v>
       </c>
     </row>
     <row r="98">
@@ -4615,7 +4615,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M98" t="str">
-        <v>2026-03-28T15:27:01.499Z</v>
+        <v>2026-03-29T15:50:37.935Z</v>
       </c>
     </row>
     <row r="99">
@@ -4656,7 +4656,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M99" t="str">
-        <v>2026-03-29T15:27:01.499Z</v>
+        <v>2026-03-30T15:50:37.935Z</v>
       </c>
     </row>
     <row r="100">
@@ -4697,7 +4697,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M100" t="str">
-        <v>2026-03-30T15:27:01.499Z</v>
+        <v>2026-03-31T15:50:37.935Z</v>
       </c>
     </row>
     <row r="101">
@@ -4738,7 +4738,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M101" t="str">
-        <v>2026-03-31T15:27:01.499Z</v>
+        <v>2026-04-01T15:50:37.935Z</v>
       </c>
     </row>
     <row r="102">
@@ -4779,7 +4779,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M102" t="str">
-        <v>2026-04-01T15:27:01.499Z</v>
+        <v>2026-04-02T15:50:37.935Z</v>
       </c>
     </row>
     <row r="103">
@@ -4820,7 +4820,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M103" t="str">
-        <v>2026-04-02T15:27:01.499Z</v>
+        <v>2026-04-03T15:50:37.935Z</v>
       </c>
     </row>
     <row r="104">
@@ -4861,7 +4861,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M104" t="str">
-        <v>2026-04-03T15:27:01.499Z</v>
+        <v>2026-04-04T15:50:37.935Z</v>
       </c>
     </row>
     <row r="105">
@@ -4902,7 +4902,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M105" t="str">
-        <v>2026-04-04T15:27:01.499Z</v>
+        <v>2026-04-05T15:50:37.935Z</v>
       </c>
     </row>
     <row r="106">
@@ -4943,7 +4943,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M106" t="str">
-        <v>2026-04-05T15:27:01.499Z</v>
+        <v>2026-04-06T15:50:37.935Z</v>
       </c>
     </row>
     <row r="107">
@@ -4984,7 +4984,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M107" t="str">
-        <v>2026-04-06T15:27:01.499Z</v>
+        <v>2026-04-07T15:50:37.935Z</v>
       </c>
     </row>
     <row r="108">
@@ -5025,7 +5025,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M108" t="str">
-        <v>2026-04-07T15:27:01.499Z</v>
+        <v>2026-04-08T15:50:37.935Z</v>
       </c>
     </row>
     <row r="109">
@@ -5066,7 +5066,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M109" t="str">
-        <v>2026-04-08T15:27:01.499Z</v>
+        <v>2026-04-09T15:50:37.935Z</v>
       </c>
     </row>
     <row r="110">
@@ -5107,7 +5107,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M110" t="str">
-        <v>2026-04-09T15:27:01.499Z</v>
+        <v>2026-04-10T15:50:37.935Z</v>
       </c>
     </row>
     <row r="111">
@@ -5148,7 +5148,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M111" t="str">
-        <v>2026-04-10T15:27:01.499Z</v>
+        <v>2026-04-11T15:50:37.935Z</v>
       </c>
     </row>
     <row r="112">
@@ -5189,7 +5189,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M112" t="str">
-        <v>2026-04-11T15:27:01.499Z</v>
+        <v>2026-04-12T15:50:37.935Z</v>
       </c>
     </row>
     <row r="113">
@@ -5230,7 +5230,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M113" t="str">
-        <v>2026-04-12T15:27:01.499Z</v>
+        <v>2026-04-13T15:50:37.935Z</v>
       </c>
     </row>
     <row r="114">
@@ -5271,7 +5271,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M114" t="str">
-        <v>2026-04-13T15:27:01.499Z</v>
+        <v>2026-04-14T15:50:37.935Z</v>
       </c>
     </row>
     <row r="115">
@@ -5312,7 +5312,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M115" t="str">
-        <v>2026-04-14T15:27:01.499Z</v>
+        <v>2026-04-15T15:50:37.935Z</v>
       </c>
     </row>
     <row r="116">
@@ -5353,7 +5353,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M116" t="str">
-        <v>2026-04-15T15:27:01.499Z</v>
+        <v>2026-04-16T15:50:37.935Z</v>
       </c>
     </row>
     <row r="117">
@@ -5394,7 +5394,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M117" t="str">
-        <v>2026-04-16T15:27:01.499Z</v>
+        <v>2026-04-17T15:50:37.935Z</v>
       </c>
     </row>
     <row r="118">
@@ -5435,7 +5435,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M118" t="str">
-        <v>2026-04-17T15:27:01.499Z</v>
+        <v>2026-04-18T15:50:37.935Z</v>
       </c>
     </row>
     <row r="119">
@@ -5476,7 +5476,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M119" t="str">
-        <v>2026-04-18T15:27:01.499Z</v>
+        <v>2026-04-19T15:50:37.935Z</v>
       </c>
     </row>
     <row r="120">
@@ -5517,7 +5517,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M120" t="str">
-        <v>2026-04-19T15:27:01.499Z</v>
+        <v>2026-04-20T15:50:37.935Z</v>
       </c>
     </row>
     <row r="121">
@@ -5558,7 +5558,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M121" t="str">
-        <v>2026-04-20T15:27:01.499Z</v>
+        <v>2026-04-21T15:50:37.935Z</v>
       </c>
     </row>
     <row r="122">
@@ -5599,7 +5599,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M122" t="str">
-        <v>2026-04-21T15:27:01.499Z</v>
+        <v>2026-04-22T15:50:37.935Z</v>
       </c>
     </row>
     <row r="123">
@@ -5640,7 +5640,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M123" t="str">
-        <v>2026-04-22T15:27:01.499Z</v>
+        <v>2026-04-23T15:50:37.935Z</v>
       </c>
     </row>
     <row r="124">
@@ -5681,7 +5681,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M124" t="str">
-        <v>2026-04-23T15:27:01.499Z</v>
+        <v>2026-04-24T15:50:37.935Z</v>
       </c>
     </row>
     <row r="125">
@@ -5722,7 +5722,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M125" t="str">
-        <v>2026-04-24T15:27:01.499Z</v>
+        <v>2026-04-25T15:50:37.935Z</v>
       </c>
     </row>
     <row r="126">
@@ -5763,7 +5763,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M126" t="str">
-        <v>2026-04-25T15:27:01.499Z</v>
+        <v>2026-04-26T15:50:37.935Z</v>
       </c>
     </row>
     <row r="127">
@@ -5804,7 +5804,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M127" t="str">
-        <v>2026-04-26T15:27:01.499Z</v>
+        <v>2026-04-27T15:50:37.935Z</v>
       </c>
     </row>
     <row r="128">
@@ -5845,7 +5845,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M128" t="str">
-        <v>2026-04-27T15:27:01.499Z</v>
+        <v>2026-04-28T15:50:37.935Z</v>
       </c>
     </row>
     <row r="129">
@@ -5886,7 +5886,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M129" t="str">
-        <v>2026-04-28T15:27:01.499Z</v>
+        <v>2026-04-29T15:50:37.935Z</v>
       </c>
     </row>
     <row r="130">
@@ -5927,7 +5927,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M130" t="str">
-        <v>2026-04-29T15:27:01.499Z</v>
+        <v>2026-04-30T15:50:37.935Z</v>
       </c>
     </row>
     <row r="131">
@@ -5968,7 +5968,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M131" t="str">
-        <v>2026-04-30T15:27:01.499Z</v>
+        <v>2026-05-01T15:50:37.935Z</v>
       </c>
     </row>
     <row r="132">
@@ -6009,7 +6009,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M132" t="str">
-        <v>2026-05-01T15:27:01.499Z</v>
+        <v>2026-05-02T15:50:37.935Z</v>
       </c>
     </row>
     <row r="133">
@@ -6050,7 +6050,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M133" t="str">
-        <v>2026-05-02T15:27:01.499Z</v>
+        <v>2026-05-03T15:50:37.935Z</v>
       </c>
     </row>
     <row r="134">
@@ -6091,7 +6091,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M134" t="str">
-        <v>2026-05-03T15:27:01.499Z</v>
+        <v>2026-05-04T15:50:37.935Z</v>
       </c>
     </row>
     <row r="135">
@@ -6132,7 +6132,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M135" t="str">
-        <v>2026-05-04T15:27:01.499Z</v>
+        <v>2026-05-05T15:50:37.935Z</v>
       </c>
     </row>
     <row r="136">
@@ -6173,7 +6173,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M136" t="str">
-        <v>2026-05-05T15:27:01.499Z</v>
+        <v>2026-05-06T15:50:37.935Z</v>
       </c>
     </row>
     <row r="137">
@@ -6214,7 +6214,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M137" t="str">
-        <v>2026-05-06T15:27:01.499Z</v>
+        <v>2026-05-07T15:50:37.935Z</v>
       </c>
     </row>
     <row r="138">
@@ -6255,7 +6255,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M138" t="str">
-        <v>2026-05-07T15:27:01.499Z</v>
+        <v>2026-05-08T15:50:37.935Z</v>
       </c>
     </row>
     <row r="139">
@@ -6296,7 +6296,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M139" t="str">
-        <v>2026-05-08T15:27:01.499Z</v>
+        <v>2026-05-09T15:50:37.935Z</v>
       </c>
     </row>
     <row r="140">
@@ -6337,7 +6337,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M140" t="str">
-        <v>2026-05-09T15:27:01.499Z</v>
+        <v>2026-05-10T15:50:37.935Z</v>
       </c>
     </row>
     <row r="141">
@@ -6378,7 +6378,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M141" t="str">
-        <v>2026-05-10T15:27:01.499Z</v>
+        <v>2026-05-11T15:50:37.935Z</v>
       </c>
     </row>
     <row r="142">
@@ -6419,7 +6419,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M142" t="str">
-        <v>2026-05-11T15:27:01.499Z</v>
+        <v>2026-05-12T15:50:37.935Z</v>
       </c>
     </row>
     <row r="143">
@@ -6460,7 +6460,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M143" t="str">
-        <v>2026-05-12T15:27:01.499Z</v>
+        <v>2026-05-13T15:50:37.935Z</v>
       </c>
     </row>
     <row r="144">
@@ -6501,7 +6501,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M144" t="str">
-        <v>2026-05-13T15:27:01.499Z</v>
+        <v>2026-05-14T15:50:37.935Z</v>
       </c>
     </row>
     <row r="145">
@@ -6542,7 +6542,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M145" t="str">
-        <v>2026-05-14T15:27:01.499Z</v>
+        <v>2026-05-15T15:50:37.935Z</v>
       </c>
     </row>
     <row r="146">
@@ -6583,7 +6583,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M146" t="str">
-        <v>2026-05-15T15:27:01.499Z</v>
+        <v>2026-05-16T15:50:37.935Z</v>
       </c>
     </row>
     <row r="147">
@@ -6624,7 +6624,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M147" t="str">
-        <v>2026-05-16T15:27:01.499Z</v>
+        <v>2026-05-17T15:50:37.935Z</v>
       </c>
     </row>
     <row r="148">
@@ -6665,7 +6665,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M148" t="str">
-        <v>2026-05-17T15:27:01.499Z</v>
+        <v>2026-05-18T15:50:37.935Z</v>
       </c>
     </row>
     <row r="149">
@@ -6706,7 +6706,7 @@
         <v>Identity verification pending.</v>
       </c>
       <c r="M149" t="str">
-        <v>2026-05-18T15:27:01.499Z</v>
+        <v>2026-05-19T15:50:37.935Z</v>
       </c>
     </row>
     <row r="150">
@@ -6747,7 +6747,7 @@
         <v>Requires compliance audit.</v>
       </c>
       <c r="M150" t="str">
-        <v>2026-05-19T15:27:01.499Z</v>
+        <v>2026-05-20T15:50:37.935Z</v>
       </c>
     </row>
     <row r="151">
@@ -6788,7 +6788,7 @@
         <v>Automated SSN &amp; Identity screening cleared.</v>
       </c>
       <c r="M151" t="str">
-        <v>2026-05-20T15:27:01.499Z</v>
+        <v>2026-05-21T15:50:37.935Z</v>
       </c>
     </row>
     <row r="152">
@@ -6829,7 +6829,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M152" t="str">
-        <v>2026-05-21T15:27:01.499Z</v>
+        <v>2026-05-22T15:50:37.935Z</v>
       </c>
     </row>
     <row r="153">
@@ -6870,7 +6870,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M153" t="str">
-        <v>2026-05-22T15:27:01.499Z</v>
+        <v>2026-05-23T15:50:37.935Z</v>
       </c>
     </row>
     <row r="154">
@@ -6911,7 +6911,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M154" t="str">
-        <v>2026-05-23T15:27:01.499Z</v>
+        <v>2026-05-24T15:50:37.935Z</v>
       </c>
     </row>
     <row r="155">
@@ -6952,7 +6952,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M155" t="str">
-        <v>2026-05-24T15:27:01.499Z</v>
+        <v>2026-05-25T15:50:37.935Z</v>
       </c>
     </row>
     <row r="156">
@@ -6993,7 +6993,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M156" t="str">
-        <v>2026-05-25T15:27:01.499Z</v>
+        <v>2026-05-26T15:50:37.935Z</v>
       </c>
     </row>
     <row r="157">
@@ -7034,7 +7034,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M157" t="str">
-        <v>2026-05-26T15:27:01.499Z</v>
+        <v>2026-05-27T15:50:37.935Z</v>
       </c>
     </row>
     <row r="158">
@@ -7075,7 +7075,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M158" t="str">
-        <v>2026-05-27T15:27:01.499Z</v>
+        <v>2026-05-28T15:50:37.935Z</v>
       </c>
     </row>
     <row r="159">
@@ -7116,7 +7116,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M159" t="str">
-        <v>2026-05-28T15:27:01.499Z</v>
+        <v>2026-05-29T15:50:37.935Z</v>
       </c>
     </row>
     <row r="160">
@@ -7157,7 +7157,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M160" t="str">
-        <v>2026-05-29T15:27:01.499Z</v>
+        <v>2026-05-30T15:50:37.935Z</v>
       </c>
     </row>
     <row r="161">
@@ -7198,7 +7198,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M161" t="str">
-        <v>2026-05-30T15:27:01.499Z</v>
+        <v>2026-05-31T15:50:37.935Z</v>
       </c>
     </row>
     <row r="162">
@@ -7239,7 +7239,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M162" t="str">
-        <v>2026-05-31T15:27:01.499Z</v>
+        <v>2026-06-01T15:50:37.935Z</v>
       </c>
     </row>
     <row r="163">
@@ -7280,7 +7280,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M163" t="str">
-        <v>2026-06-01T15:27:01.499Z</v>
+        <v>2026-06-02T15:50:37.935Z</v>
       </c>
     </row>
     <row r="164">
@@ -7321,7 +7321,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M164" t="str">
-        <v>2026-06-02T15:27:01.499Z</v>
+        <v>2026-06-03T15:50:37.935Z</v>
       </c>
     </row>
     <row r="165">
@@ -7362,7 +7362,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M165" t="str">
-        <v>2026-06-03T15:27:01.499Z</v>
+        <v>2026-06-04T15:50:37.935Z</v>
       </c>
     </row>
     <row r="166">
@@ -7403,7 +7403,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M166" t="str">
-        <v>2026-06-04T15:27:01.499Z</v>
+        <v>2026-06-05T15:50:37.935Z</v>
       </c>
     </row>
     <row r="167">
@@ -7444,7 +7444,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M167" t="str">
-        <v>2026-06-05T15:27:01.499Z</v>
+        <v>2026-06-06T15:50:37.935Z</v>
       </c>
     </row>
     <row r="168">
@@ -7485,7 +7485,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M168" t="str">
-        <v>2026-06-06T15:27:01.499Z</v>
+        <v>2026-06-07T15:50:37.935Z</v>
       </c>
     </row>
     <row r="169">
@@ -7526,7 +7526,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M169" t="str">
-        <v>2026-06-07T15:27:01.499Z</v>
+        <v>2026-06-08T15:50:37.935Z</v>
       </c>
     </row>
     <row r="170">
@@ -7567,7 +7567,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M170" t="str">
-        <v>2026-06-08T15:27:01.499Z</v>
+        <v>2026-06-09T15:50:37.935Z</v>
       </c>
     </row>
     <row r="171">
@@ -7608,7 +7608,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M171" t="str">
-        <v>2026-06-09T15:27:01.499Z</v>
+        <v>2026-06-10T15:50:37.935Z</v>
       </c>
     </row>
     <row r="172">
@@ -7649,7 +7649,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M172" t="str">
-        <v>2026-06-10T15:27:01.499Z</v>
+        <v>2026-06-11T15:50:37.935Z</v>
       </c>
     </row>
     <row r="173">
@@ -7690,7 +7690,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M173" t="str">
-        <v>2026-06-11T15:27:01.499Z</v>
+        <v>2026-06-12T15:50:37.935Z</v>
       </c>
     </row>
     <row r="174">
@@ -7731,7 +7731,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M174" t="str">
-        <v>2026-06-12T15:27:01.499Z</v>
+        <v>2026-06-13T15:50:37.935Z</v>
       </c>
     </row>
     <row r="175">
@@ -7772,7 +7772,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M175" t="str">
-        <v>2026-06-13T15:27:01.499Z</v>
+        <v>2026-06-14T15:50:37.935Z</v>
       </c>
     </row>
     <row r="176">
@@ -7813,7 +7813,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M176" t="str">
-        <v>2026-06-14T15:27:01.499Z</v>
+        <v>2026-06-15T15:50:37.935Z</v>
       </c>
     </row>
     <row r="177">
@@ -7854,7 +7854,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M177" t="str">
-        <v>2026-06-15T15:27:01.499Z</v>
+        <v>2026-06-16T15:50:37.935Z</v>
       </c>
     </row>
     <row r="178">
@@ -7895,7 +7895,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M178" t="str">
-        <v>2026-06-16T15:27:01.499Z</v>
+        <v>2026-06-17T15:50:37.935Z</v>
       </c>
     </row>
     <row r="179">
@@ -7936,7 +7936,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M179" t="str">
-        <v>2026-06-17T15:27:01.499Z</v>
+        <v>2026-06-18T15:50:37.935Z</v>
       </c>
     </row>
     <row r="180">
@@ -7977,7 +7977,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M180" t="str">
-        <v>2026-06-18T15:27:01.499Z</v>
+        <v>2026-06-19T15:50:37.935Z</v>
       </c>
     </row>
     <row r="181">
@@ -8018,7 +8018,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M181" t="str">
-        <v>2026-06-19T15:27:01.499Z</v>
+        <v>2026-06-20T15:50:37.935Z</v>
       </c>
     </row>
     <row r="182">
@@ -8059,7 +8059,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M182" t="str">
-        <v>2026-06-20T15:27:01.499Z</v>
+        <v>2026-06-21T15:50:37.935Z</v>
       </c>
     </row>
     <row r="183">
@@ -8100,7 +8100,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M183" t="str">
-        <v>2026-06-21T15:27:01.499Z</v>
+        <v>2026-06-22T15:50:37.935Z</v>
       </c>
     </row>
     <row r="184">
@@ -8141,7 +8141,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M184" t="str">
-        <v>2026-06-22T15:27:01.499Z</v>
+        <v>2026-06-23T15:50:37.935Z</v>
       </c>
     </row>
     <row r="185">
@@ -8182,7 +8182,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M185" t="str">
-        <v>2026-06-23T15:27:01.499Z</v>
+        <v>2026-06-24T15:50:37.935Z</v>
       </c>
     </row>
     <row r="186">
@@ -8223,7 +8223,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M186" t="str">
-        <v>2026-06-24T15:27:01.499Z</v>
+        <v>2026-06-25T15:50:37.935Z</v>
       </c>
     </row>
     <row r="187">
@@ -8264,7 +8264,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M187" t="str">
-        <v>2026-06-25T15:27:01.499Z</v>
+        <v>2026-06-26T15:50:37.935Z</v>
       </c>
     </row>
     <row r="188">
@@ -8305,7 +8305,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M188" t="str">
-        <v>2026-06-26T15:27:01.499Z</v>
+        <v>2026-06-27T15:50:37.935Z</v>
       </c>
     </row>
     <row r="189">
@@ -8346,7 +8346,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M189" t="str">
-        <v>2026-06-27T15:27:01.499Z</v>
+        <v>2026-06-28T15:50:37.935Z</v>
       </c>
     </row>
     <row r="190">
@@ -8387,7 +8387,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M190" t="str">
-        <v>2026-06-28T15:27:01.499Z</v>
+        <v>2026-06-29T15:50:37.935Z</v>
       </c>
     </row>
     <row r="191">
@@ -8428,7 +8428,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M191" t="str">
-        <v>2026-06-29T15:27:01.499Z</v>
+        <v>2026-06-30T15:50:37.935Z</v>
       </c>
     </row>
     <row r="192">
@@ -8469,7 +8469,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M192" t="str">
-        <v>2026-06-30T15:27:01.499Z</v>
+        <v>2026-07-01T15:50:37.935Z</v>
       </c>
     </row>
     <row r="193">
@@ -8510,7 +8510,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M193" t="str">
-        <v>2026-07-01T15:27:01.499Z</v>
+        <v>2026-07-02T15:50:37.935Z</v>
       </c>
     </row>
     <row r="194">
@@ -8551,7 +8551,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M194" t="str">
-        <v>2026-07-02T15:27:01.499Z</v>
+        <v>2026-07-03T15:50:37.935Z</v>
       </c>
     </row>
     <row r="195">
@@ -8592,7 +8592,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M195" t="str">
-        <v>2026-07-03T15:27:01.499Z</v>
+        <v>2026-07-04T15:50:37.935Z</v>
       </c>
     </row>
     <row r="196">
@@ -8633,7 +8633,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M196" t="str">
-        <v>2026-07-04T15:27:01.499Z</v>
+        <v>2026-07-05T15:50:37.935Z</v>
       </c>
     </row>
     <row r="197">
@@ -8674,7 +8674,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M197" t="str">
-        <v>2026-07-05T15:27:01.499Z</v>
+        <v>2026-07-06T15:50:37.935Z</v>
       </c>
     </row>
     <row r="198">
@@ -8715,7 +8715,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M198" t="str">
-        <v>2026-07-06T15:27:01.499Z</v>
+        <v>2026-07-07T15:50:37.935Z</v>
       </c>
     </row>
     <row r="199">
@@ -8756,7 +8756,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M199" t="str">
-        <v>2026-07-07T15:27:01.499Z</v>
+        <v>2026-07-08T15:50:37.935Z</v>
       </c>
     </row>
     <row r="200">
@@ -8797,7 +8797,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M200" t="str">
-        <v>2026-07-08T15:27:01.499Z</v>
+        <v>2026-07-09T15:50:37.935Z</v>
       </c>
     </row>
     <row r="201">
@@ -8838,7 +8838,7 @@
         <v>High-Net-Worth Private Wealth Clearance.</v>
       </c>
       <c r="M201" t="str">
-        <v>2026-07-09T15:27:01.499Z</v>
+        <v>2026-07-10T15:50:37.935Z</v>
       </c>
     </row>
     <row r="202">
@@ -8879,7 +8879,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M202" t="str">
-        <v>2026-07-10T15:27:01.499Z</v>
+        <v>2026-07-11T15:50:37.936Z</v>
       </c>
     </row>
     <row r="203">
@@ -8920,7 +8920,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M203" t="str">
-        <v>2026-07-11T15:27:01.499Z</v>
+        <v>2026-07-12T15:50:37.936Z</v>
       </c>
     </row>
     <row r="204">
@@ -8961,7 +8961,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M204" t="str">
-        <v>2026-07-12T15:27:01.499Z</v>
+        <v>2026-07-13T15:50:37.936Z</v>
       </c>
     </row>
     <row r="205">
@@ -9002,7 +9002,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M205" t="str">
-        <v>2026-07-13T15:27:01.499Z</v>
+        <v>2026-07-14T15:50:37.936Z</v>
       </c>
     </row>
     <row r="206">
@@ -9043,7 +9043,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M206" t="str">
-        <v>2026-07-14T15:27:01.499Z</v>
+        <v>2026-07-15T15:50:37.936Z</v>
       </c>
     </row>
     <row r="207">
@@ -9084,7 +9084,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M207" t="str">
-        <v>2026-07-15T15:27:01.500Z</v>
+        <v>2026-07-16T15:50:37.936Z</v>
       </c>
     </row>
     <row r="208">
@@ -9125,7 +9125,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M208" t="str">
-        <v>2026-07-16T15:27:01.500Z</v>
+        <v>2026-07-17T15:50:37.936Z</v>
       </c>
     </row>
     <row r="209">
@@ -9166,7 +9166,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M209" t="str">
-        <v>2026-07-17T15:27:01.500Z</v>
+        <v>2026-07-18T15:50:37.936Z</v>
       </c>
     </row>
     <row r="210">
@@ -9207,7 +9207,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M210" t="str">
-        <v>2026-07-18T15:27:01.500Z</v>
+        <v>2026-07-19T15:50:37.936Z</v>
       </c>
     </row>
     <row r="211">
@@ -9248,7 +9248,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M211" t="str">
-        <v>2026-07-19T15:27:01.500Z</v>
+        <v>2026-07-20T15:50:37.936Z</v>
       </c>
     </row>
     <row r="212">
@@ -9289,7 +9289,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M212" t="str">
-        <v>2026-07-20T15:27:01.500Z</v>
+        <v>2026-07-21T15:50:37.936Z</v>
       </c>
     </row>
     <row r="213">
@@ -9330,7 +9330,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M213" t="str">
-        <v>2026-07-21T15:27:01.500Z</v>
+        <v>2026-07-22T15:50:37.936Z</v>
       </c>
     </row>
     <row r="214">
@@ -9371,7 +9371,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M214" t="str">
-        <v>2026-07-22T15:27:01.500Z</v>
+        <v>2026-07-23T15:50:37.936Z</v>
       </c>
     </row>
     <row r="215">
@@ -9412,7 +9412,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M215" t="str">
-        <v>2026-07-23T15:27:01.500Z</v>
+        <v>2026-07-24T15:50:37.936Z</v>
       </c>
     </row>
     <row r="216">
@@ -9453,7 +9453,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M216" t="str">
-        <v>2026-07-24T15:27:01.500Z</v>
+        <v>2026-07-25T15:50:37.936Z</v>
       </c>
     </row>
     <row r="217">
@@ -9494,7 +9494,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M217" t="str">
-        <v>2026-07-25T15:27:01.500Z</v>
+        <v>2026-07-26T15:50:37.936Z</v>
       </c>
     </row>
     <row r="218">
@@ -9535,7 +9535,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M218" t="str">
-        <v>2026-07-26T15:27:01.500Z</v>
+        <v>2026-07-27T15:50:37.936Z</v>
       </c>
     </row>
     <row r="219">
@@ -9576,7 +9576,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M219" t="str">
-        <v>2026-07-27T15:27:01.500Z</v>
+        <v>2026-07-28T15:50:37.936Z</v>
       </c>
     </row>
     <row r="220">
@@ -9617,7 +9617,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M220" t="str">
-        <v>2026-07-28T15:27:01.500Z</v>
+        <v>2026-07-29T15:50:37.936Z</v>
       </c>
     </row>
     <row r="221">
@@ -9658,7 +9658,7 @@
         <v>Corporate Beneficial Ownership cleared.</v>
       </c>
       <c r="M221" t="str">
-        <v>2026-07-29T15:27:01.500Z</v>
+        <v>2026-07-30T15:50:37.936Z</v>
       </c>
     </row>
   </sheetData>
@@ -9709,378 +9709,378 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>c0000001-1111-4111-c111-111111111111</v>
+        <v>c0000042-1111-4111-c111-111111111111</v>
       </c>
       <c r="B2" t="str">
-        <v>b0000001-1111-4111-b111-111111111111</v>
+        <v>b0000042-1111-4111-b111-111111111111</v>
       </c>
       <c r="C2" t="str">
-        <v>Alexander Chen</v>
+        <v>N/A</v>
       </c>
       <c r="D2" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E2">
-        <v>400000</v>
+        <v>8080000</v>
       </c>
       <c r="F2">
-        <v>4.5</v>
+        <v>5.25</v>
       </c>
       <c r="G2">
-        <v>12</v>
+        <v>240</v>
       </c>
       <c r="H2" t="str">
-        <v>Equipment Purchase &amp; Automation</v>
+        <v>Estate Development &amp; High Net-Worth Credit</v>
       </c>
       <c r="I2" t="str">
-        <v>draft</v>
+        <v>rejected</v>
       </c>
       <c r="J2">
         <v>94</v>
       </c>
       <c r="K2" t="str">
-        <v>2026-07-02T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>c0000002-1111-4111-c111-111111111111</v>
+        <v>c0000041-1111-4111-c111-111111111111</v>
       </c>
       <c r="B3" t="str">
-        <v>b0000002-1111-4111-b111-111111111111</v>
+        <v>b0000041-1111-4111-b111-111111111111</v>
       </c>
       <c r="C3" t="str">
-        <v>Sarah Green</v>
+        <v>N/A</v>
       </c>
       <c r="D3" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E3">
-        <v>880000</v>
+        <v>7600000</v>
       </c>
       <c r="F3">
-        <v>5.25</v>
+        <v>4.5</v>
       </c>
       <c r="G3">
-        <v>24</v>
+        <v>120</v>
       </c>
       <c r="H3" t="str">
-        <v>Working Capital Expansion</v>
+        <v>Personal Wealth Portfolio Scaling</v>
       </c>
       <c r="I3" t="str">
-        <v>compliance_review</v>
+        <v>disbursed</v>
       </c>
       <c r="J3">
         <v>94</v>
       </c>
       <c r="K3" t="str">
-        <v>2026-07-03T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>c0000003-1111-4111-c111-111111111111</v>
+        <v>c0000049-1111-4111-c111-111111111111</v>
       </c>
       <c r="B4" t="str">
-        <v>b0000003-1111-4111-b111-111111111111</v>
+        <v>b0000049-1111-4111-b111-111111111111</v>
       </c>
       <c r="C4" t="str">
-        <v>David Reddy</v>
+        <v>N/A</v>
       </c>
       <c r="D4" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E4">
-        <v>1360000</v>
+        <v>11440000</v>
       </c>
       <c r="F4">
-        <v>6</v>
+        <v>4.5</v>
       </c>
       <c r="G4">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="H4" t="str">
-        <v>Commercial Real Estate Acquisition</v>
+        <v>Estate Development &amp; High Net-Worth Credit</v>
       </c>
       <c r="I4" t="str">
         <v>underwriting</v>
       </c>
       <c r="J4">
-        <v>94</v>
+        <v>35</v>
       </c>
       <c r="K4" t="str">
-        <v>2026-07-03T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>c0000004-1111-4111-c111-111111111111</v>
+        <v>c0000043-1111-4111-c111-111111111111</v>
       </c>
       <c r="B5" t="str">
-        <v>b0000004-1111-4111-b111-111111111111</v>
+        <v>b0000043-1111-4111-b111-111111111111</v>
       </c>
       <c r="C5" t="str">
-        <v>Elena Smith</v>
+        <v>N/A</v>
       </c>
       <c r="D5" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E5">
-        <v>1840000</v>
+        <v>8560000</v>
       </c>
       <c r="F5">
-        <v>6.75</v>
+        <v>6</v>
       </c>
       <c r="G5">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="H5" t="str">
-        <v>Debt Refinancing &amp; Consolidation</v>
+        <v>Equipment Purchase &amp; Automation</v>
       </c>
       <c r="I5" t="str">
-        <v>approved</v>
+        <v>underwriting</v>
       </c>
       <c r="J5">
-        <v>94</v>
+        <v>35</v>
       </c>
       <c r="K5" t="str">
-        <v>2026-07-04T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>c0000005-1111-4111-c111-111111111111</v>
+        <v>c0000054-1111-4111-c111-111111111111</v>
       </c>
       <c r="B6" t="str">
-        <v>b0000005-1111-4111-b111-111111111111</v>
+        <v>b0000054-1111-4111-b111-111111111111</v>
       </c>
       <c r="C6" t="str">
-        <v>Marcus Jones</v>
+        <v>N/A</v>
       </c>
       <c r="D6" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E6">
-        <v>2320000</v>
+        <v>1840000</v>
       </c>
       <c r="F6">
-        <v>7.5</v>
+        <v>8.25</v>
       </c>
       <c r="G6">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="H6" t="str">
         <v>R&amp;D Facility Upgrade</v>
       </c>
       <c r="I6" t="str">
-        <v>disbursed</v>
+        <v>rejected</v>
       </c>
       <c r="J6">
-        <v>94</v>
+        <v>36</v>
       </c>
       <c r="K6" t="str">
-        <v>2026-07-04T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>c0000006-1111-4111-c111-111111111111</v>
+        <v>c0000053-1111-4111-c111-111111111111</v>
       </c>
       <c r="B7" t="str">
-        <v>b0000006-1111-4111-b111-111111111111</v>
+        <v>b0000053-1111-4111-b111-111111111111</v>
       </c>
       <c r="C7" t="str">
-        <v>Rachel Davis</v>
+        <v>N/A</v>
       </c>
       <c r="D7" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E7">
-        <v>2800000</v>
+        <v>1360000</v>
       </c>
       <c r="F7">
-        <v>8.25</v>
+        <v>7.5</v>
       </c>
       <c r="G7">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="H7" t="str">
-        <v>Personal Wealth Portfolio Scaling</v>
+        <v>Debt Refinancing &amp; Consolidation</v>
       </c>
       <c r="I7" t="str">
-        <v>rejected</v>
+        <v>disbursed</v>
       </c>
       <c r="J7">
-        <v>94</v>
+        <v>32</v>
       </c>
       <c r="K7" t="str">
-        <v>2026-07-05T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>c0000007-1111-4111-c111-111111111111</v>
+        <v>c0000052-1111-4111-c111-111111111111</v>
       </c>
       <c r="B8" t="str">
-        <v>b0000007-1111-4111-b111-111111111111</v>
+        <v>b0000052-1111-4111-b111-111111111111</v>
       </c>
       <c r="C8" t="str">
-        <v>Vikram Hernandez</v>
+        <v>N/A</v>
       </c>
       <c r="D8" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E8">
-        <v>3280000</v>
+        <v>880000</v>
       </c>
       <c r="F8">
-        <v>9</v>
+        <v>6.75</v>
       </c>
       <c r="G8">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="H8" t="str">
-        <v>Estate Development &amp; High Net-Worth Credit</v>
+        <v>Commercial Real Estate Acquisition</v>
       </c>
       <c r="I8" t="str">
-        <v>draft</v>
+        <v>approved</v>
       </c>
       <c r="J8">
-        <v>94</v>
+        <v>28</v>
       </c>
       <c r="K8" t="str">
-        <v>2026-07-05T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>c0000008-1111-4111-c111-111111111111</v>
+        <v>c0000051-1111-4111-c111-111111111111</v>
       </c>
       <c r="B9" t="str">
-        <v>b0000008-1111-4111-b111-111111111111</v>
+        <v>b0000051-1111-4111-b111-111111111111</v>
       </c>
       <c r="C9" t="str">
-        <v>Priya Wilson</v>
+        <v>N/A</v>
       </c>
       <c r="D9" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E9">
-        <v>3760000</v>
+        <v>400000</v>
       </c>
       <c r="F9">
-        <v>9.75</v>
+        <v>6</v>
       </c>
       <c r="G9">
+        <v>36</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Working Capital Expansion</v>
+      </c>
+      <c r="I9" t="str">
+        <v>underwriting</v>
+      </c>
+      <c r="J9">
         <v>24</v>
       </c>
-      <c r="H9" t="str">
-        <v>Equipment Purchase &amp; Automation</v>
-      </c>
-      <c r="I9" t="str">
-        <v>compliance_review</v>
-      </c>
-      <c r="J9">
-        <v>94</v>
-      </c>
       <c r="K9" t="str">
-        <v>2026-07-06T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>c0000009-1111-4111-c111-111111111111</v>
+        <v>c0000050-1111-4111-c111-111111111111</v>
       </c>
       <c r="B10" t="str">
-        <v>b0000009-1111-4111-b111-111111111111</v>
+        <v>b0000050-1111-4111-b111-111111111111</v>
       </c>
       <c r="C10" t="str">
-        <v>Ananya Taylor</v>
+        <v>N/A</v>
       </c>
       <c r="D10" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E10">
-        <v>4240000</v>
+        <v>11920000</v>
       </c>
       <c r="F10">
-        <v>4.5</v>
+        <v>5.25</v>
       </c>
       <c r="G10">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="H10" t="str">
-        <v>Working Capital Expansion</v>
+        <v>Equipment Purchase &amp; Automation</v>
       </c>
       <c r="I10" t="str">
-        <v>underwriting</v>
+        <v>compliance_review</v>
       </c>
       <c r="J10">
         <v>94</v>
       </c>
       <c r="K10" t="str">
-        <v>2026-07-06T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>c0000010-1111-4111-c111-111111111111</v>
+        <v>c0000048-1111-4111-c111-111111111111</v>
       </c>
       <c r="B11" t="str">
-        <v>b0000010-1111-4111-b111-111111111111</v>
+        <v>b0000048-1111-4111-b111-111111111111</v>
       </c>
       <c r="C11" t="str">
-        <v>Rohan Martin</v>
+        <v>N/A</v>
       </c>
       <c r="D11" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E11">
-        <v>4720000</v>
+        <v>10960000</v>
       </c>
       <c r="F11">
-        <v>5.25</v>
+        <v>9.75</v>
       </c>
       <c r="G11">
-        <v>60</v>
+        <v>240</v>
       </c>
       <c r="H11" t="str">
-        <v>Commercial Real Estate Acquisition</v>
+        <v>Personal Wealth Portfolio Scaling</v>
       </c>
       <c r="I11" t="str">
-        <v>approved</v>
+        <v>rejected</v>
       </c>
       <c r="J11">
         <v>94</v>
       </c>
       <c r="K11" t="str">
-        <v>2026-07-07T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>c0000011-1111-4111-c111-111111111111</v>
+        <v>c0000047-1111-4111-c111-111111111111</v>
       </c>
       <c r="B12" t="str">
-        <v>b0000011-1111-4111-b111-111111111111</v>
+        <v>b0000047-1111-4111-b111-111111111111</v>
       </c>
       <c r="C12" t="str">
-        <v>Michael Thompson</v>
+        <v>N/A</v>
       </c>
       <c r="D12" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E12">
-        <v>5200000</v>
+        <v>10480000</v>
       </c>
       <c r="F12">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G12">
         <v>120</v>
       </c>
       <c r="H12" t="str">
-        <v>Debt Refinancing &amp; Consolidation</v>
+        <v>R&amp;D Facility Upgrade</v>
       </c>
       <c r="I12" t="str">
         <v>disbursed</v>
@@ -10089,103 +10089,103 @@
         <v>94</v>
       </c>
       <c r="K12" t="str">
-        <v>2026-07-07T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>c0000012-1111-4111-c111-111111111111</v>
+        <v>c0000046-1111-4111-c111-111111111111</v>
       </c>
       <c r="B13" t="str">
-        <v>b0000012-1111-4111-b111-111111111111</v>
+        <v>b0000046-1111-4111-b111-111111111111</v>
       </c>
       <c r="C13" t="str">
-        <v>Jessica Sanchez</v>
+        <v>N/A</v>
       </c>
       <c r="D13" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E13">
-        <v>5680000</v>
+        <v>10000000</v>
       </c>
       <c r="F13">
-        <v>6.75</v>
+        <v>8.25</v>
       </c>
       <c r="G13">
-        <v>240</v>
+        <v>60</v>
       </c>
       <c r="H13" t="str">
-        <v>R&amp;D Facility Upgrade</v>
+        <v>Debt Refinancing &amp; Consolidation</v>
       </c>
       <c r="I13" t="str">
-        <v>rejected</v>
+        <v>approved</v>
       </c>
       <c r="J13">
         <v>94</v>
       </c>
       <c r="K13" t="str">
-        <v>2026-07-08T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>c0000013-1111-4111-c111-111111111111</v>
+        <v>c0000045-1111-4111-c111-111111111111</v>
       </c>
       <c r="B14" t="str">
-        <v>b0000013-1111-4111-b111-111111111111</v>
+        <v>b0000045-1111-4111-b111-111111111111</v>
       </c>
       <c r="C14" t="str">
-        <v>Emily Lewis</v>
+        <v>N/A</v>
       </c>
       <c r="D14" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E14">
-        <v>6160000</v>
+        <v>9520000</v>
       </c>
       <c r="F14">
         <v>7.5</v>
       </c>
       <c r="G14">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="H14" t="str">
-        <v>Personal Wealth Portfolio Scaling</v>
+        <v>Commercial Real Estate Acquisition</v>
       </c>
       <c r="I14" t="str">
-        <v>draft</v>
+        <v>underwriting</v>
       </c>
       <c r="J14">
         <v>94</v>
       </c>
       <c r="K14" t="str">
-        <v>2026-07-08T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>c0000014-1111-4111-c111-111111111111</v>
+        <v>c0000044-1111-4111-c111-111111111111</v>
       </c>
       <c r="B15" t="str">
-        <v>b0000014-1111-4111-b111-111111111111</v>
+        <v>b0000044-1111-4111-b111-111111111111</v>
       </c>
       <c r="C15" t="str">
-        <v>Christopher Jenkins</v>
+        <v>N/A</v>
       </c>
       <c r="D15" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E15">
-        <v>6640000</v>
+        <v>9040000</v>
       </c>
       <c r="F15">
-        <v>8.25</v>
+        <v>6.75</v>
       </c>
       <c r="G15">
         <v>24</v>
       </c>
       <c r="H15" t="str">
-        <v>Estate Development &amp; High Net-Worth Credit</v>
+        <v>Working Capital Expansion</v>
       </c>
       <c r="I15" t="str">
         <v>compliance_review</v>
@@ -10194,838 +10194,838 @@
         <v>94</v>
       </c>
       <c r="K15" t="str">
-        <v>2026-07-09T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.912599+00:00</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>c0000015-1111-4111-c111-111111111111</v>
+        <v>c0000028-1111-4111-c111-111111111111</v>
       </c>
       <c r="B16" t="str">
-        <v>b0000015-1111-4111-b111-111111111111</v>
+        <v>b0000028-1111-4111-b111-111111111111</v>
       </c>
       <c r="C16" t="str">
-        <v>Amanda Vance</v>
+        <v>N/A</v>
       </c>
       <c r="D16" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E16">
-        <v>7120000</v>
+        <v>1360000</v>
       </c>
       <c r="F16">
-        <v>9</v>
+        <v>6.75</v>
       </c>
       <c r="G16">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="H16" t="str">
-        <v>Equipment Purchase &amp; Automation</v>
+        <v>Estate Development &amp; High Net-Worth Credit</v>
       </c>
       <c r="I16" t="str">
-        <v>underwriting</v>
+        <v>approved</v>
       </c>
       <c r="J16">
-        <v>94</v>
+        <v>42</v>
       </c>
       <c r="K16" t="str">
-        <v>2026-07-09T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>c0000016-1111-4111-c111-111111111111</v>
+        <v>c0000022-1111-4111-c111-111111111111</v>
       </c>
       <c r="B17" t="str">
-        <v>b0000016-1111-4111-b111-111111111111</v>
+        <v>b0000022-1111-4111-b111-111111111111</v>
       </c>
       <c r="C17" t="str">
-        <v>Daniel Patel</v>
+        <v>N/A</v>
       </c>
       <c r="D17" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E17">
-        <v>7600000</v>
+        <v>10480000</v>
       </c>
       <c r="F17">
-        <v>9.75</v>
+        <v>8.25</v>
       </c>
       <c r="G17">
         <v>60</v>
       </c>
       <c r="H17" t="str">
-        <v>Working Capital Expansion</v>
+        <v>Equipment Purchase &amp; Automation</v>
       </c>
       <c r="I17" t="str">
-        <v>approved</v>
+        <v>disbursed</v>
       </c>
       <c r="J17">
         <v>94</v>
       </c>
       <c r="K17" t="str">
-        <v>2026-07-10T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>c0000017-1111-4111-c111-111111111111</v>
+        <v>c0000030-1111-4111-c111-111111111111</v>
       </c>
       <c r="B18" t="str">
-        <v>b0000017-1111-4111-b111-111111111111</v>
+        <v>b0000030-1111-4111-b111-111111111111</v>
       </c>
       <c r="C18" t="str">
-        <v>Sophia Johnson</v>
+        <v>N/A</v>
       </c>
       <c r="D18" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E18">
-        <v>8080000</v>
+        <v>2320000</v>
       </c>
       <c r="F18">
-        <v>4.5</v>
+        <v>8.25</v>
       </c>
       <c r="G18">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="H18" t="str">
-        <v>Commercial Real Estate Acquisition</v>
+        <v>Working Capital Expansion</v>
       </c>
       <c r="I18" t="str">
-        <v>disbursed</v>
+        <v>rejected</v>
       </c>
       <c r="J18">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="K18" t="str">
-        <v>2026-07-10T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>c0000018-1111-4111-c111-111111111111</v>
+        <v>c0000038-1111-4111-c111-111111111111</v>
       </c>
       <c r="B19" t="str">
-        <v>b0000018-1111-4111-b111-111111111111</v>
+        <v>b0000038-1111-4111-b111-111111111111</v>
       </c>
       <c r="C19" t="str">
-        <v>James Brown</v>
+        <v>N/A</v>
       </c>
       <c r="D19" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E19">
-        <v>8560000</v>
+        <v>6160000</v>
       </c>
       <c r="F19">
-        <v>5.25</v>
+        <v>8.25</v>
       </c>
       <c r="G19">
-        <v>240</v>
+        <v>24</v>
       </c>
       <c r="H19" t="str">
-        <v>Debt Refinancing &amp; Consolidation</v>
+        <v>Commercial Real Estate Acquisition</v>
       </c>
       <c r="I19" t="str">
-        <v>rejected</v>
+        <v>compliance_review</v>
       </c>
       <c r="J19">
         <v>94</v>
       </c>
       <c r="K19" t="str">
-        <v>2026-07-11T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>c0000019-1111-4111-c111-111111111111</v>
+        <v>c0000039-1111-4111-c111-111111111111</v>
       </c>
       <c r="B20" t="str">
-        <v>b0000019-1111-4111-b111-111111111111</v>
+        <v>b0000039-1111-4111-b111-111111111111</v>
       </c>
       <c r="C20" t="str">
-        <v>Olivia Miller</v>
+        <v>N/A</v>
       </c>
       <c r="D20" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E20">
-        <v>9040000</v>
+        <v>6640000</v>
       </c>
       <c r="F20">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G20">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="H20" t="str">
-        <v>R&amp;D Facility Upgrade</v>
+        <v>Debt Refinancing &amp; Consolidation</v>
       </c>
       <c r="I20" t="str">
-        <v>draft</v>
+        <v>underwriting</v>
       </c>
       <c r="J20">
         <v>94</v>
       </c>
       <c r="K20" t="str">
-        <v>2026-07-11T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>c0000020-1111-4111-c111-111111111111</v>
+        <v>c0000029-1111-4111-c111-111111111111</v>
       </c>
       <c r="B21" t="str">
-        <v>b0000020-1111-4111-b111-111111111111</v>
+        <v>b0000029-1111-4111-b111-111111111111</v>
       </c>
       <c r="C21" t="str">
-        <v>Ethan Martinez</v>
+        <v>N/A</v>
       </c>
       <c r="D21" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E21">
-        <v>9520000</v>
+        <v>1840000</v>
       </c>
       <c r="F21">
-        <v>6.75</v>
+        <v>7.5</v>
       </c>
       <c r="G21">
-        <v>24</v>
+        <v>120</v>
       </c>
       <c r="H21" t="str">
-        <v>Personal Wealth Portfolio Scaling</v>
+        <v>Equipment Purchase &amp; Automation</v>
       </c>
       <c r="I21" t="str">
-        <v>compliance_review</v>
+        <v>disbursed</v>
       </c>
       <c r="J21">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="K21" t="str">
-        <v>2026-07-12T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>c0000021-1111-4111-c111-111111111111</v>
+        <v>c0000034-1111-4111-c111-111111111111</v>
       </c>
       <c r="B22" t="str">
-        <v>b0000021-1111-4111-b111-111111111111</v>
+        <v>b0000034-1111-4111-b111-111111111111</v>
       </c>
       <c r="C22" t="str">
-        <v>Isabella Gonzalez</v>
+        <v>N/A</v>
       </c>
       <c r="D22" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E22">
-        <v>10000000</v>
+        <v>4240000</v>
       </c>
       <c r="F22">
-        <v>7.5</v>
+        <v>5.25</v>
       </c>
       <c r="G22">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="H22" t="str">
-        <v>Estate Development &amp; High Net-Worth Credit</v>
+        <v>Personal Wealth Portfolio Scaling</v>
       </c>
       <c r="I22" t="str">
-        <v>underwriting</v>
+        <v>approved</v>
       </c>
       <c r="J22">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="K22" t="str">
-        <v>2026-07-12T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>c0000022-1111-4111-c111-111111111111</v>
+        <v>c0000023-1111-4111-c111-111111111111</v>
       </c>
       <c r="B23" t="str">
-        <v>b0000022-1111-4111-b111-111111111111</v>
+        <v>b0000023-1111-4111-b111-111111111111</v>
       </c>
       <c r="C23" t="str">
-        <v>William Thomas</v>
+        <v>N/A</v>
       </c>
       <c r="D23" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E23">
-        <v>10480000</v>
+        <v>10960000</v>
       </c>
       <c r="F23">
-        <v>8.25</v>
+        <v>9</v>
       </c>
       <c r="G23">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="H23" t="str">
-        <v>Equipment Purchase &amp; Automation</v>
+        <v>Working Capital Expansion</v>
       </c>
       <c r="I23" t="str">
-        <v>approved</v>
+        <v>disbursed</v>
       </c>
       <c r="J23">
         <v>94</v>
       </c>
       <c r="K23" t="str">
-        <v>2026-07-13T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>c0000023-1111-4111-c111-111111111111</v>
+        <v>c0000024-1111-4111-c111-111111111111</v>
       </c>
       <c r="B24" t="str">
-        <v>b0000023-1111-4111-b111-111111111111</v>
+        <v>b0000024-1111-4111-b111-111111111111</v>
       </c>
       <c r="C24" t="str">
-        <v>Ava Jackson</v>
+        <v>N/A</v>
       </c>
       <c r="D24" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E24">
-        <v>10960000</v>
+        <v>11440000</v>
       </c>
       <c r="F24">
-        <v>9</v>
+        <v>9.75</v>
       </c>
       <c r="G24">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="H24" t="str">
-        <v>Working Capital Expansion</v>
+        <v>Commercial Real Estate Acquisition</v>
       </c>
       <c r="I24" t="str">
-        <v>disbursed</v>
+        <v>rejected</v>
       </c>
       <c r="J24">
         <v>94</v>
       </c>
       <c r="K24" t="str">
-        <v>2026-07-13T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>c0000024-1111-4111-c111-111111111111</v>
+        <v>c0000025-1111-4111-c111-111111111111</v>
       </c>
       <c r="B25" t="str">
-        <v>b0000024-1111-4111-b111-111111111111</v>
+        <v>b0000025-1111-4111-b111-111111111111</v>
       </c>
       <c r="C25" t="str">
-        <v>Benjamin Perez</v>
+        <v>N/A</v>
       </c>
       <c r="D25" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E25">
-        <v>11440000</v>
+        <v>11920000</v>
       </c>
       <c r="F25">
-        <v>9.75</v>
+        <v>4.5</v>
       </c>
       <c r="G25">
-        <v>240</v>
+        <v>12</v>
       </c>
       <c r="H25" t="str">
-        <v>Commercial Real Estate Acquisition</v>
+        <v>Debt Refinancing &amp; Consolidation</v>
       </c>
       <c r="I25" t="str">
-        <v>rejected</v>
+        <v>draft</v>
       </c>
       <c r="J25">
         <v>94</v>
       </c>
       <c r="K25" t="str">
-        <v>2026-07-14T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>c0000025-1111-4111-c111-111111111111</v>
+        <v>c0000026-1111-4111-c111-111111111111</v>
       </c>
       <c r="B26" t="str">
-        <v>b0000025-1111-4111-b111-111111111111</v>
+        <v>b0000026-1111-4111-b111-111111111111</v>
       </c>
       <c r="C26" t="str">
-        <v>Mia Harris</v>
+        <v>N/A</v>
       </c>
       <c r="D26" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E26">
-        <v>11920000</v>
+        <v>400000</v>
       </c>
       <c r="F26">
-        <v>4.5</v>
+        <v>5.25</v>
       </c>
       <c r="G26">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="H26" t="str">
-        <v>Debt Refinancing &amp; Consolidation</v>
+        <v>R&amp;D Facility Upgrade</v>
       </c>
       <c r="I26" t="str">
-        <v>draft</v>
+        <v>compliance_review</v>
       </c>
       <c r="J26">
-        <v>94</v>
+        <v>27</v>
       </c>
       <c r="K26" t="str">
-        <v>2026-07-14T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>c0000026-1111-4111-c111-111111111111</v>
+        <v>c0000031-1111-4111-c111-111111111111</v>
       </c>
       <c r="B27" t="str">
-        <v>b0000026-1111-4111-b111-111111111111</v>
+        <v>b0000031-1111-4111-b111-111111111111</v>
       </c>
       <c r="C27" t="str">
-        <v>Lucas Ramirez</v>
+        <v>N/A</v>
       </c>
       <c r="D27" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E27">
-        <v>400000</v>
+        <v>2800000</v>
       </c>
       <c r="F27">
-        <v>5.25</v>
+        <v>9</v>
       </c>
       <c r="G27">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H27" t="str">
-        <v>R&amp;D Facility Upgrade</v>
+        <v>Commercial Real Estate Acquisition</v>
       </c>
       <c r="I27" t="str">
-        <v>compliance_review</v>
+        <v>draft</v>
       </c>
       <c r="J27">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="K27" t="str">
-        <v>2026-07-15T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>c0000027-1111-4111-c111-111111111111</v>
+        <v>c0000032-1111-4111-c111-111111111111</v>
       </c>
       <c r="B28" t="str">
-        <v>b0000027-1111-4111-b111-111111111111</v>
+        <v>b0000032-1111-4111-b111-111111111111</v>
       </c>
       <c r="C28" t="str">
-        <v>Charlotte Sterling</v>
+        <v>N/A</v>
       </c>
       <c r="D28" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E28">
-        <v>880000</v>
+        <v>3280000</v>
       </c>
       <c r="F28">
-        <v>6</v>
+        <v>9.75</v>
       </c>
       <c r="G28">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="H28" t="str">
-        <v>Personal Wealth Portfolio Scaling</v>
+        <v>Debt Refinancing &amp; Consolidation</v>
       </c>
       <c r="I28" t="str">
-        <v>underwriting</v>
+        <v>compliance_review</v>
       </c>
       <c r="J28">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="K28" t="str">
-        <v>2026-07-15T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>c0000028-1111-4111-c111-111111111111</v>
+        <v>c0000033-1111-4111-c111-111111111111</v>
       </c>
       <c r="B29" t="str">
-        <v>b0000028-1111-4111-b111-111111111111</v>
+        <v>b0000033-1111-4111-b111-111111111111</v>
       </c>
       <c r="C29" t="str">
-        <v>Henry Rostova</v>
+        <v>N/A</v>
       </c>
       <c r="D29" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E29">
-        <v>1360000</v>
+        <v>3760000</v>
       </c>
       <c r="F29">
-        <v>6.75</v>
+        <v>4.5</v>
       </c>
       <c r="G29">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="H29" t="str">
-        <v>Estate Development &amp; High Net-Worth Credit</v>
+        <v>R&amp;D Facility Upgrade</v>
       </c>
       <c r="I29" t="str">
-        <v>approved</v>
+        <v>underwriting</v>
       </c>
       <c r="J29">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="K29" t="str">
-        <v>2026-07-16T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>c0000029-1111-4111-c111-111111111111</v>
+        <v>c0000035-1111-4111-c111-111111111111</v>
       </c>
       <c r="B30" t="str">
-        <v>b0000029-1111-4111-b111-111111111111</v>
+        <v>b0000035-1111-4111-b111-111111111111</v>
       </c>
       <c r="C30" t="str">
-        <v>Amelia Sharma</v>
+        <v>N/A</v>
       </c>
       <c r="D30" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E30">
-        <v>1840000</v>
+        <v>4720000</v>
       </c>
       <c r="F30">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G30">
         <v>120</v>
       </c>
       <c r="H30" t="str">
-        <v>Equipment Purchase &amp; Automation</v>
+        <v>Estate Development &amp; High Net-Worth Credit</v>
       </c>
       <c r="I30" t="str">
         <v>disbursed</v>
       </c>
       <c r="J30">
-        <v>49</v>
+        <v>83</v>
       </c>
       <c r="K30" t="str">
-        <v>2026-07-16T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>c0000030-1111-4111-c111-111111111111</v>
+        <v>c0000036-1111-4111-c111-111111111111</v>
       </c>
       <c r="B31" t="str">
-        <v>b0000030-1111-4111-b111-111111111111</v>
+        <v>b0000036-1111-4111-b111-111111111111</v>
       </c>
       <c r="C31" t="str">
-        <v>Alexander Mehta</v>
+        <v>N/A</v>
       </c>
       <c r="D31" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E31">
-        <v>2320000</v>
+        <v>5200000</v>
       </c>
       <c r="F31">
-        <v>8.25</v>
+        <v>6.75</v>
       </c>
       <c r="G31">
         <v>240</v>
       </c>
       <c r="H31" t="str">
-        <v>Working Capital Expansion</v>
+        <v>Equipment Purchase &amp; Automation</v>
       </c>
       <c r="I31" t="str">
         <v>rejected</v>
       </c>
       <c r="J31">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="K31" t="str">
-        <v>2026-07-17T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>c0000031-1111-4111-c111-111111111111</v>
+        <v>c0000037-1111-4111-c111-111111111111</v>
       </c>
       <c r="B32" t="str">
-        <v>b0000031-1111-4111-b111-111111111111</v>
+        <v>b0000037-1111-4111-b111-111111111111</v>
       </c>
       <c r="C32" t="str">
-        <v>Harper Williams</v>
+        <v>N/A</v>
       </c>
       <c r="D32" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E32">
-        <v>2800000</v>
+        <v>5680000</v>
       </c>
       <c r="F32">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="G32">
         <v>12</v>
       </c>
       <c r="H32" t="str">
-        <v>Commercial Real Estate Acquisition</v>
+        <v>Working Capital Expansion</v>
       </c>
       <c r="I32" t="str">
         <v>draft</v>
       </c>
       <c r="J32">
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="K32" t="str">
-        <v>2026-07-17T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>c0000032-1111-4111-c111-111111111111</v>
+        <v>c0000021-1111-4111-c111-111111111111</v>
       </c>
       <c r="B33" t="str">
-        <v>b0000032-1111-4111-b111-111111111111</v>
+        <v>b0000021-1111-4111-b111-111111111111</v>
       </c>
       <c r="C33" t="str">
-        <v>Sebastian Garcia</v>
+        <v>N/A</v>
       </c>
       <c r="D33" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E33">
-        <v>3280000</v>
+        <v>10000000</v>
       </c>
       <c r="F33">
-        <v>9.75</v>
+        <v>7.5</v>
       </c>
       <c r="G33">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="H33" t="str">
-        <v>Debt Refinancing &amp; Consolidation</v>
+        <v>Estate Development &amp; High Net-Worth Credit</v>
       </c>
       <c r="I33" t="str">
-        <v>compliance_review</v>
+        <v>underwriting</v>
       </c>
       <c r="J33">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="K33" t="str">
-        <v>2026-07-18T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>c0000033-1111-4111-c111-111111111111</v>
+        <v>c0000027-1111-4111-c111-111111111111</v>
       </c>
       <c r="B34" t="str">
-        <v>b0000033-1111-4111-b111-111111111111</v>
+        <v>b0000027-1111-4111-b111-111111111111</v>
       </c>
       <c r="C34" t="str">
-        <v>Evelyn Rodriguez</v>
+        <v>N/A</v>
       </c>
       <c r="D34" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E34">
-        <v>3760000</v>
+        <v>880000</v>
       </c>
       <c r="F34">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="G34">
         <v>36</v>
       </c>
       <c r="H34" t="str">
-        <v>R&amp;D Facility Upgrade</v>
+        <v>Personal Wealth Portfolio Scaling</v>
       </c>
       <c r="I34" t="str">
         <v>underwriting</v>
       </c>
       <c r="J34">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="K34" t="str">
-        <v>2026-07-18T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.735094+00:00</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>c0000034-1111-4111-c111-111111111111</v>
+        <v>c0000018-1111-4111-c111-111111111111</v>
       </c>
       <c r="B35" t="str">
-        <v>b0000034-1111-4111-b111-111111111111</v>
+        <v>b0000018-1111-4111-b111-111111111111</v>
       </c>
       <c r="C35" t="str">
-        <v>Jack Lopez</v>
+        <v>N/A</v>
       </c>
       <c r="D35" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E35">
-        <v>4240000</v>
+        <v>8560000</v>
       </c>
       <c r="F35">
         <v>5.25</v>
       </c>
       <c r="G35">
-        <v>60</v>
+        <v>240</v>
       </c>
       <c r="H35" t="str">
-        <v>Personal Wealth Portfolio Scaling</v>
+        <v>Debt Refinancing &amp; Consolidation</v>
       </c>
       <c r="I35" t="str">
-        <v>approved</v>
+        <v>rejected</v>
       </c>
       <c r="J35">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="K35" t="str">
-        <v>2026-07-19T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>c0000035-1111-4111-c111-111111111111</v>
+        <v>c0000005-1111-4111-c111-111111111111</v>
       </c>
       <c r="B36" t="str">
-        <v>b0000035-1111-4111-b111-111111111111</v>
+        <v>b0000005-1111-4111-b111-111111111111</v>
       </c>
       <c r="C36" t="str">
-        <v>Abigail Anderson</v>
+        <v>N/A</v>
       </c>
       <c r="D36" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E36">
-        <v>4720000</v>
+        <v>2320000</v>
       </c>
       <c r="F36">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G36">
         <v>120</v>
       </c>
       <c r="H36" t="str">
-        <v>Estate Development &amp; High Net-Worth Credit</v>
+        <v>R&amp;D Facility Upgrade</v>
       </c>
       <c r="I36" t="str">
         <v>disbursed</v>
       </c>
       <c r="J36">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="K36" t="str">
-        <v>2026-07-19T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>c0000036-1111-4111-c111-111111111111</v>
+        <v>c0000004-1111-4111-c111-111111111111</v>
       </c>
       <c r="B37" t="str">
-        <v>b0000036-1111-4111-b111-111111111111</v>
+        <v>b0000004-1111-4111-b111-111111111111</v>
       </c>
       <c r="C37" t="str">
-        <v>Owen Moore</v>
+        <v>N/A</v>
       </c>
       <c r="D37" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E37">
-        <v>5200000</v>
+        <v>1840000</v>
       </c>
       <c r="F37">
         <v>6.75</v>
       </c>
       <c r="G37">
-        <v>240</v>
+        <v>60</v>
       </c>
       <c r="H37" t="str">
-        <v>Equipment Purchase &amp; Automation</v>
+        <v>Debt Refinancing &amp; Consolidation</v>
       </c>
       <c r="I37" t="str">
-        <v>rejected</v>
+        <v>approved</v>
       </c>
       <c r="J37">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="K37" t="str">
-        <v>2026-07-20T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>c0000037-1111-4111-c111-111111111111</v>
+        <v>c0000003-1111-4111-c111-111111111111</v>
       </c>
       <c r="B38" t="str">
-        <v>b0000037-1111-4111-b111-111111111111</v>
+        <v>b0000003-1111-4111-b111-111111111111</v>
       </c>
       <c r="C38" t="str">
-        <v>Emily Lee</v>
+        <v>N/A</v>
       </c>
       <c r="D38" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E38">
-        <v>5680000</v>
+        <v>1360000</v>
       </c>
       <c r="F38">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G38">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="H38" t="str">
-        <v>Working Capital Expansion</v>
+        <v>Commercial Real Estate Acquisition</v>
       </c>
       <c r="I38" t="str">
-        <v>draft</v>
+        <v>underwriting</v>
       </c>
       <c r="J38">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="K38" t="str">
-        <v>2026-07-20T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>c0000038-1111-4111-c111-111111111111</v>
+        <v>c0000002-1111-4111-c111-111111111111</v>
       </c>
       <c r="B39" t="str">
-        <v>b0000038-1111-4111-b111-111111111111</v>
+        <v>b0000002-1111-4111-b111-111111111111</v>
       </c>
       <c r="C39" t="str">
-        <v>Theodore White</v>
+        <v>N/A</v>
       </c>
       <c r="D39" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E39">
-        <v>6160000</v>
+        <v>880000</v>
       </c>
       <c r="F39">
-        <v>8.25</v>
+        <v>5.25</v>
       </c>
       <c r="G39">
         <v>24</v>
       </c>
       <c r="H39" t="str">
-        <v>Commercial Real Estate Acquisition</v>
+        <v>Working Capital Expansion</v>
       </c>
       <c r="I39" t="str">
         <v>compliance_review</v>
@@ -11034,164 +11034,164 @@
         <v>94</v>
       </c>
       <c r="K39" t="str">
-        <v>2026-07-21T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>c0000039-1111-4111-c111-111111111111</v>
+        <v>c0000001-1111-4111-c111-111111111111</v>
       </c>
       <c r="B40" t="str">
-        <v>b0000039-1111-4111-b111-111111111111</v>
+        <v>b0000001-1111-4111-b111-111111111111</v>
       </c>
       <c r="C40" t="str">
-        <v>Ella Clark</v>
+        <v>N/A</v>
       </c>
       <c r="D40" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E40">
-        <v>6640000</v>
+        <v>400000</v>
       </c>
       <c r="F40">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="G40">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="H40" t="str">
-        <v>Debt Refinancing &amp; Consolidation</v>
+        <v>Equipment Purchase &amp; Automation</v>
       </c>
       <c r="I40" t="str">
-        <v>underwriting</v>
+        <v>draft</v>
       </c>
       <c r="J40">
         <v>94</v>
       </c>
       <c r="K40" t="str">
-        <v>2026-07-21T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>c0000040-1111-4111-c111-111111111111</v>
+        <v>c0000009-1111-4111-c111-111111111111</v>
       </c>
       <c r="B41" t="str">
-        <v>b0000040-1111-4111-b111-111111111111</v>
+        <v>b0000009-1111-4111-b111-111111111111</v>
       </c>
       <c r="C41" t="str">
-        <v>Katherapaka Srinivas</v>
+        <v>N/A</v>
       </c>
       <c r="D41" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E41">
-        <v>7120000</v>
+        <v>4240000</v>
       </c>
       <c r="F41">
-        <v>9.75</v>
+        <v>4.5</v>
       </c>
       <c r="G41">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="H41" t="str">
-        <v>R&amp;D Facility Upgrade</v>
+        <v>Working Capital Expansion</v>
       </c>
       <c r="I41" t="str">
-        <v>approved</v>
+        <v>underwriting</v>
       </c>
       <c r="J41">
         <v>94</v>
       </c>
       <c r="K41" t="str">
-        <v>2026-07-22T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>c0000041-1111-4111-c111-111111111111</v>
+        <v>c0000015-1111-4111-c111-111111111111</v>
       </c>
       <c r="B42" t="str">
-        <v>b0000041-1111-4111-b111-111111111111</v>
+        <v>b0000015-1111-4111-b111-111111111111</v>
       </c>
       <c r="C42" t="str">
-        <v>Alexander Chen</v>
+        <v>N/A</v>
       </c>
       <c r="D42" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E42">
-        <v>7600000</v>
+        <v>7120000</v>
       </c>
       <c r="F42">
-        <v>4.5</v>
+        <v>9</v>
       </c>
       <c r="G42">
-        <v>120</v>
+        <v>36</v>
       </c>
       <c r="H42" t="str">
-        <v>Personal Wealth Portfolio Scaling</v>
+        <v>Equipment Purchase &amp; Automation</v>
       </c>
       <c r="I42" t="str">
-        <v>disbursed</v>
+        <v>underwriting</v>
       </c>
       <c r="J42">
         <v>94</v>
       </c>
       <c r="K42" t="str">
-        <v>2026-07-22T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>c0000042-1111-4111-c111-111111111111</v>
+        <v>c0000016-1111-4111-c111-111111111111</v>
       </c>
       <c r="B43" t="str">
-        <v>b0000042-1111-4111-b111-111111111111</v>
+        <v>b0000016-1111-4111-b111-111111111111</v>
       </c>
       <c r="C43" t="str">
-        <v>Sarah Green</v>
+        <v>N/A</v>
       </c>
       <c r="D43" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E43">
-        <v>8080000</v>
+        <v>7600000</v>
       </c>
       <c r="F43">
-        <v>5.25</v>
+        <v>9.75</v>
       </c>
       <c r="G43">
-        <v>240</v>
+        <v>60</v>
       </c>
       <c r="H43" t="str">
-        <v>Estate Development &amp; High Net-Worth Credit</v>
+        <v>Working Capital Expansion</v>
       </c>
       <c r="I43" t="str">
-        <v>rejected</v>
+        <v>approved</v>
       </c>
       <c r="J43">
         <v>94</v>
       </c>
       <c r="K43" t="str">
-        <v>2026-07-23T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>c0000043-1111-4111-c111-111111111111</v>
+        <v>c0000019-1111-4111-c111-111111111111</v>
       </c>
       <c r="B44" t="str">
-        <v>b0000043-1111-4111-b111-111111111111</v>
+        <v>b0000019-1111-4111-b111-111111111111</v>
       </c>
       <c r="C44" t="str">
-        <v>David Reddy</v>
+        <v>N/A</v>
       </c>
       <c r="D44" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E44">
-        <v>8560000</v>
+        <v>9040000</v>
       </c>
       <c r="F44">
         <v>6</v>
@@ -11200,7 +11200,7 @@
         <v>12</v>
       </c>
       <c r="H44" t="str">
-        <v>Equipment Purchase &amp; Automation</v>
+        <v>R&amp;D Facility Upgrade</v>
       </c>
       <c r="I44" t="str">
         <v>draft</v>
@@ -11209,24 +11209,24 @@
         <v>94</v>
       </c>
       <c r="K44" t="str">
-        <v>2026-07-23T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>c0000044-1111-4111-c111-111111111111</v>
+        <v>c0000020-1111-4111-c111-111111111111</v>
       </c>
       <c r="B45" t="str">
-        <v>b0000044-1111-4111-b111-111111111111</v>
+        <v>b0000020-1111-4111-b111-111111111111</v>
       </c>
       <c r="C45" t="str">
-        <v>Elena Smith</v>
+        <v>N/A</v>
       </c>
       <c r="D45" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E45">
-        <v>9040000</v>
+        <v>9520000</v>
       </c>
       <c r="F45">
         <v>6.75</v>
@@ -11235,7 +11235,7 @@
         <v>24</v>
       </c>
       <c r="H45" t="str">
-        <v>Working Capital Expansion</v>
+        <v>Personal Wealth Portfolio Scaling</v>
       </c>
       <c r="I45" t="str">
         <v>compliance_review</v>
@@ -11244,103 +11244,103 @@
         <v>94</v>
       </c>
       <c r="K45" t="str">
-        <v>2026-07-24T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>c0000045-1111-4111-c111-111111111111</v>
+        <v>c0000014-1111-4111-c111-111111111111</v>
       </c>
       <c r="B46" t="str">
-        <v>b0000045-1111-4111-b111-111111111111</v>
+        <v>b0000014-1111-4111-b111-111111111111</v>
       </c>
       <c r="C46" t="str">
-        <v>Marcus Jones</v>
+        <v>N/A</v>
       </c>
       <c r="D46" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E46">
-        <v>9520000</v>
+        <v>6640000</v>
       </c>
       <c r="F46">
-        <v>7.5</v>
+        <v>8.25</v>
       </c>
       <c r="G46">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="H46" t="str">
-        <v>Commercial Real Estate Acquisition</v>
+        <v>Estate Development &amp; High Net-Worth Credit</v>
       </c>
       <c r="I46" t="str">
-        <v>underwriting</v>
+        <v>compliance_review</v>
       </c>
       <c r="J46">
         <v>94</v>
       </c>
       <c r="K46" t="str">
-        <v>2026-07-24T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>c0000046-1111-4111-c111-111111111111</v>
+        <v>c0000013-1111-4111-c111-111111111111</v>
       </c>
       <c r="B47" t="str">
-        <v>b0000046-1111-4111-b111-111111111111</v>
+        <v>b0000013-1111-4111-b111-111111111111</v>
       </c>
       <c r="C47" t="str">
-        <v>Rachel Davis</v>
+        <v>N/A</v>
       </c>
       <c r="D47" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E47">
-        <v>10000000</v>
+        <v>6160000</v>
       </c>
       <c r="F47">
-        <v>8.25</v>
+        <v>7.5</v>
       </c>
       <c r="G47">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="H47" t="str">
-        <v>Debt Refinancing &amp; Consolidation</v>
+        <v>Personal Wealth Portfolio Scaling</v>
       </c>
       <c r="I47" t="str">
-        <v>approved</v>
+        <v>draft</v>
       </c>
       <c r="J47">
         <v>94</v>
       </c>
       <c r="K47" t="str">
-        <v>2026-07-25T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>c0000047-1111-4111-c111-111111111111</v>
+        <v>c0000017-1111-4111-c111-111111111111</v>
       </c>
       <c r="B48" t="str">
-        <v>b0000047-1111-4111-b111-111111111111</v>
+        <v>b0000017-1111-4111-b111-111111111111</v>
       </c>
       <c r="C48" t="str">
-        <v>Vikram Hernandez</v>
+        <v>N/A</v>
       </c>
       <c r="D48" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E48">
-        <v>10480000</v>
+        <v>8080000</v>
       </c>
       <c r="F48">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="G48">
         <v>120</v>
       </c>
       <c r="H48" t="str">
-        <v>R&amp;D Facility Upgrade</v>
+        <v>Commercial Real Estate Acquisition</v>
       </c>
       <c r="I48" t="str">
         <v>disbursed</v>
@@ -11349,27 +11349,27 @@
         <v>94</v>
       </c>
       <c r="K48" t="str">
-        <v>2026-07-25T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>c0000048-1111-4111-c111-111111111111</v>
+        <v>c0000006-1111-4111-c111-111111111111</v>
       </c>
       <c r="B49" t="str">
-        <v>b0000048-1111-4111-b111-111111111111</v>
+        <v>b0000006-1111-4111-b111-111111111111</v>
       </c>
       <c r="C49" t="str">
-        <v>Priya Wilson</v>
+        <v>N/A</v>
       </c>
       <c r="D49" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E49">
-        <v>10960000</v>
+        <v>2800000</v>
       </c>
       <c r="F49">
-        <v>9.75</v>
+        <v>8.25</v>
       </c>
       <c r="G49">
         <v>240</v>
@@ -11384,217 +11384,217 @@
         <v>94</v>
       </c>
       <c r="K49" t="str">
-        <v>2026-07-26T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>c0000049-1111-4111-c111-111111111111</v>
+        <v>c0000012-1111-4111-c111-111111111111</v>
       </c>
       <c r="B50" t="str">
-        <v>b0000049-1111-4111-b111-111111111111</v>
+        <v>b0000012-1111-4111-b111-111111111111</v>
       </c>
       <c r="C50" t="str">
-        <v>Ananya Taylor</v>
+        <v>N/A</v>
       </c>
       <c r="D50" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E50">
-        <v>11440000</v>
+        <v>5680000</v>
       </c>
       <c r="F50">
-        <v>4.5</v>
+        <v>6.75</v>
       </c>
       <c r="G50">
-        <v>12</v>
+        <v>240</v>
       </c>
       <c r="H50" t="str">
-        <v>Estate Development &amp; High Net-Worth Credit</v>
+        <v>R&amp;D Facility Upgrade</v>
       </c>
       <c r="I50" t="str">
-        <v>draft</v>
+        <v>rejected</v>
       </c>
       <c r="J50">
         <v>94</v>
       </c>
       <c r="K50" t="str">
-        <v>2026-07-26T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>c0000050-1111-4111-c111-111111111111</v>
+        <v>c0000011-1111-4111-c111-111111111111</v>
       </c>
       <c r="B51" t="str">
-        <v>b0000050-1111-4111-b111-111111111111</v>
+        <v>b0000011-1111-4111-b111-111111111111</v>
       </c>
       <c r="C51" t="str">
-        <v>Rohan Martin</v>
+        <v>N/A</v>
       </c>
       <c r="D51" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E51">
-        <v>11920000</v>
+        <v>5200000</v>
       </c>
       <c r="F51">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="G51">
-        <v>24</v>
+        <v>120</v>
       </c>
       <c r="H51" t="str">
-        <v>Equipment Purchase &amp; Automation</v>
+        <v>Debt Refinancing &amp; Consolidation</v>
       </c>
       <c r="I51" t="str">
-        <v>compliance_review</v>
+        <v>disbursed</v>
       </c>
       <c r="J51">
         <v>94</v>
       </c>
       <c r="K51" t="str">
-        <v>2026-07-27T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>c0000051-1111-4111-c111-111111111111</v>
+        <v>c0000010-1111-4111-c111-111111111111</v>
       </c>
       <c r="B52" t="str">
-        <v>b0000051-1111-4111-b111-111111111111</v>
+        <v>b0000010-1111-4111-b111-111111111111</v>
       </c>
       <c r="C52" t="str">
-        <v>Michael Thompson</v>
+        <v>N/A</v>
       </c>
       <c r="D52" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E52">
-        <v>400000</v>
+        <v>4720000</v>
       </c>
       <c r="F52">
-        <v>6</v>
+        <v>5.25</v>
       </c>
       <c r="G52">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="H52" t="str">
-        <v>Working Capital Expansion</v>
+        <v>Commercial Real Estate Acquisition</v>
       </c>
       <c r="I52" t="str">
-        <v>underwriting</v>
+        <v>approved</v>
       </c>
       <c r="J52">
-        <v>24</v>
+        <v>94</v>
       </c>
       <c r="K52" t="str">
-        <v>2026-07-27T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>c0000052-1111-4111-c111-111111111111</v>
+        <v>c0000008-1111-4111-c111-111111111111</v>
       </c>
       <c r="B53" t="str">
-        <v>b0000052-1111-4111-b111-111111111111</v>
+        <v>b0000008-1111-4111-b111-111111111111</v>
       </c>
       <c r="C53" t="str">
-        <v>Jessica Sanchez</v>
+        <v>N/A</v>
       </c>
       <c r="D53" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E53">
-        <v>880000</v>
+        <v>3760000</v>
       </c>
       <c r="F53">
-        <v>6.75</v>
+        <v>9.75</v>
       </c>
       <c r="G53">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="H53" t="str">
-        <v>Commercial Real Estate Acquisition</v>
+        <v>Equipment Purchase &amp; Automation</v>
       </c>
       <c r="I53" t="str">
-        <v>approved</v>
+        <v>compliance_review</v>
       </c>
       <c r="J53">
-        <v>28</v>
+        <v>94</v>
       </c>
       <c r="K53" t="str">
-        <v>2026-07-28T03:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>c0000053-1111-4111-c111-111111111111</v>
+        <v>c0000007-1111-4111-c111-111111111111</v>
       </c>
       <c r="B54" t="str">
-        <v>b0000053-1111-4111-b111-111111111111</v>
+        <v>b0000007-1111-4111-b111-111111111111</v>
       </c>
       <c r="C54" t="str">
-        <v>Emily Lewis</v>
+        <v>N/A</v>
       </c>
       <c r="D54" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E54">
-        <v>1360000</v>
+        <v>3280000</v>
       </c>
       <c r="F54">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="G54">
-        <v>120</v>
+        <v>12</v>
       </c>
       <c r="H54" t="str">
-        <v>Debt Refinancing &amp; Consolidation</v>
+        <v>Estate Development &amp; High Net-Worth Credit</v>
       </c>
       <c r="I54" t="str">
-        <v>disbursed</v>
+        <v>draft</v>
       </c>
       <c r="J54">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="K54" t="str">
-        <v>2026-07-28T15:27:01.500Z</v>
+        <v>2026-07-29T15:27:02.612077+00:00</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>c0000054-1111-4111-c111-111111111111</v>
+        <v>c1111111-1111-4111-c111-111111111111</v>
       </c>
       <c r="B55" t="str">
-        <v>b0000054-1111-4111-b111-111111111111</v>
+        <v>b1111111-1111-4111-b111-111111111111</v>
       </c>
       <c r="C55" t="str">
-        <v>Christopher Jenkins</v>
+        <v>N/A</v>
       </c>
       <c r="D55" t="str">
-        <v>private_savings</v>
+        <v>N/A</v>
       </c>
       <c r="E55">
-        <v>1840000</v>
+        <v>2500000</v>
       </c>
       <c r="F55">
-        <v>8.25</v>
+        <v>6.5</v>
       </c>
       <c r="G55">
-        <v>240</v>
+        <v>36</v>
       </c>
       <c r="H55" t="str">
-        <v>R&amp;D Facility Upgrade</v>
+        <v>Equipment Purchase &amp; Factory Expansion</v>
       </c>
       <c r="I55" t="str">
-        <v>rejected</v>
+        <v>disbursed</v>
       </c>
       <c r="J55">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="K55" t="str">
-        <v>2026-07-29T03:27:01.500Z</v>
+        <v>2026-07-29T09:10:43.491177+00:00</v>
       </c>
     </row>
   </sheetData>
@@ -11639,7 +11639,7 @@
         <v>50000000</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-07-29T15:27:01.496Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="3">
@@ -11656,7 +11656,7 @@
         <v>0</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-07-29T15:27:01.497Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="4">
@@ -11673,7 +11673,7 @@
         <v>50000000</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-07-29T15:27:01.497Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="5">
@@ -11690,7 +11690,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-07-29T15:27:01.497Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="6">
@@ -11707,7 +11707,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-07-29T15:27:01.497Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
   </sheetData>
@@ -11719,7 +11719,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11743,7 +11743,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>e2c9b4e2-ae19-4458-84af-003c0204870f</v>
+        <v>v1000001-1111-4111-v111-111111111111</v>
       </c>
       <c r="B2" t="str">
         <v>Global Tech Hardware Inc</v>
@@ -11758,12 +11758,12 @@
         <v>Approved</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-07-29T15:27:01.497Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>69e5615d-99c3-49ff-86fb-0500c1b13ec6</v>
+        <v>v1000002-2222-4222-v222-222222222222</v>
       </c>
       <c r="B3" t="str">
         <v>CyberShield Banking Security</v>
@@ -11778,12 +11778,12 @@
         <v>Approved</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-07-29T15:27:01.497Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>761bf11c-7a2a-46fc-a73e-287ad0c44a13</v>
+        <v>v1000003-3333-4333-v333-333333333333</v>
       </c>
       <c r="B4" t="str">
         <v>OmniCloud Data Infrastructure</v>
@@ -11798,12 +11798,112 @@
         <v>Approved</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-07-29T15:27:01.497Z</v>
+        <v>2026-07-30T15:50:37.934Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>v1000004-4444-4444-v444-444444444444</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Apex Data Center Solutions</v>
+      </c>
+      <c r="C5" t="str">
+        <v>US-7711005</v>
+      </c>
+      <c r="D5" t="str">
+        <v>orders@apexdatacenters.com</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-07-30T15:50:37.934Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>v1000005-5555-4555-v555-555555555555</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Vanguard ATM &amp; Vault Hardware</v>
+      </c>
+      <c r="C6" t="str">
+        <v>US-3344556</v>
+      </c>
+      <c r="D6" t="str">
+        <v>finance@vanguardatm.com</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-07-30T15:50:37.934Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>v1000006-6666-4666-v666-666666666666</v>
+      </c>
+      <c r="B7" t="str">
+        <v>BioPharma Commercial Equipment</v>
+      </c>
+      <c r="C7" t="str">
+        <v>US-6655443</v>
+      </c>
+      <c r="D7" t="str">
+        <v>accounts@biopharmasupplies.com</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-07-30T15:50:37.934Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>v1000007-7777-4777-v777-777777777777</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Titan Real Estate Management</v>
+      </c>
+      <c r="C8" t="str">
+        <v>US-2233441</v>
+      </c>
+      <c r="D8" t="str">
+        <v>billing@titanproperties.com</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-07-30T15:50:37.934Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>v1000008-8888-4888-v888-888888888888</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Solstice Renewable Energy Corp</v>
+      </c>
+      <c r="C9" t="str">
+        <v>US-1122334</v>
+      </c>
+      <c r="D9" t="str">
+        <v>orders@solsticepower.com</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-07-30T15:50:37.934Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>